<commit_message>
Validation kit: call script, outreach messages, target farms
- docs/validation/call-script.en.md and .ar.md: a 30-minute call built
  on questions about past behaviour, a demo walkthrough, the free
  3-month pilot offer, common objections and a scorecard. The Arabic
  is Modern Standard Arabic.
- docs/validation/outreach-messages.md: WhatsApp, LinkedIn and email
  messages in English and Arabic (first touch, follow-up, last note,
  partner version, quick replies), using the spreadsheet's placeholders.
- docs/validation/target-farms.md: 22 organisations in Jordan, the UAE
  and Saudi Arabia from public sources, with priority, fit, first
  channel, language and a source link for each.
- docs/outreach-links.xlsx: prefilled with the 22 targets. Messages
  read naturally when the contact name is still blank.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dm6j71QsxSkbatZyu95Fda
</commit_message>
<xml_diff>
--- a/docs/outreach-links.xlsx
+++ b/docs/outreach-links.xlsx
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="89">
   <si>
     <t xml:space="preserve">Canopy outreach links</t>
   </si>
@@ -138,28 +138,163 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">Green Valley Farms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Omar</t>
+    <t xml:space="preserve">iPlant</t>
   </si>
   <si>
     <t xml:space="preserve">Jordan</t>
   </si>
   <si>
-    <t xml:space="preserve">+962 7 9000 0000</t>
+    <t xml:space="preserve">linkedin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A · urban/vertical farming systems, Amman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypo-Farm</t>
   </si>
   <si>
     <t xml:space="preserve">whatsapp</t>
   </si>
   <si>
+    <t xml:space="preserve">A · hydroponic herb farm, Amman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smart Green</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C · IoT sensor partner, Irbid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECO Consult</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email</t>
+  </si>
+  <si>
     <t xml:space="preserve">en</t>
   </si>
   <si>
-    <t xml:space="preserve">to contact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example row: replace or delete</t>
+    <t xml:space="preserve">C · hydroponic programmes, many farms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HAED-Jo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C · hydroponics programme, farm directory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NARC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C · national research centre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B · women-led hydroponic cooperative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Badia Farms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A · vertical microgreens, Dubai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Madar Farms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A · container + indoor tomatoes, Abu Dhabi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emirates Hydroponics Farms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A · hydroponic grower since 2005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VeggiTech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B · builds/operates hydroponic farms; check Dubai vs Sharjah entity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emirates Bustanica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B · very large vertical farm; later, with a pilot to show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pure Harvest Smart Farms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B · GCC greenhouses; later, with a pilot to show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iFarm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C · vertical farm tech supplier, partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C · research centre, Dubai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bather Smart Farm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saudi Arabia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A · vertical leafy greens, Riyadh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mojan Farms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A · hydroponic greenhouses, Jeddah (Instagram)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertical Farms Company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B · Mowreq + YesHealth JV; confirm it's open</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RedSea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C · hot-climate greenhouse tech, partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAUST Center for Desert Agriculture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C · research centre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KACST Green CEA Centre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desert Agriculture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B · verify active first, Dammam</t>
   </si>
   <si>
     <t xml:space="preserve">How to use this sheet</t>
@@ -168,7 +303,7 @@
     <t xml:space="preserve">1. Set the site address and campaign name at the top of the Links tab (yellow cells).</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Add one farm per row: farm name, contact's first name, country, phone, channel and language (en or ar).</t>
+    <t xml:space="preserve">2. 22 target farms are already listed (see docs/validation/target-farms.md). Add the contact's first name and phone, or add new farms below.</t>
   </si>
   <si>
     <t xml:space="preserve">3. The demo link, message and WhatsApp link fill in on their own. Click "Send on WhatsApp" to open a chat with the message ready.</t>
@@ -853,523 +988,771 @@
       <c r="A10" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7"/>
+      <c r="E10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="F10" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>31</v>
       </c>
       <c r="G10" s="8" t="str">
         <f aca="false">IF(A10="","",$B$4&amp;"/"&amp;IF(F10="","en",F10)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A10)&amp;"&amp;utm_source="&amp;IF(E10="","direct",E10)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-1")</f>
-        <v>https://your-domain.com/en/demo?farm=Green%20Valley%20Farms&amp;utm_source=whatsapp&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-1</v>
+        <v>https://your-domain.com/ar/demo?farm=iPlant&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-1</v>
       </c>
       <c r="H10" s="9" t="str">
-        <f aca="false">IF(A10="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F10="ar",$B$7,$B$6),"{name}",IF(B10="","",B10)),"{farm}",A10),"{link}",G10))</f>
-        <v>Hi Omar, I made a live 3D demo of Green Valley Farms so you can see how it would look: https://your-domain.com/en/demo?farm=Green%20Valley%20Farms&amp;utm_source=whatsapp&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-1  Would you be open to a 30-minute call this week?</v>
+        <f aca="false">IF(A10="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F10="ar",$B$7,$B$6)," {name}",IF(B10="",""," "&amp;B10)),"{farm}",A10),"{link}",G10))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ iPlant لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=iPlant&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-1  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I10" s="9" t="str">
         <f aca="false">IF(OR(A10="",D10=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D10,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H10),"Send on WhatsApp"))</f>
-        <v>Send on WhatsApp</v>
+        <v/>
       </c>
       <c r="J10" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K10" s="10"/>
       <c r="L10" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="F11" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G11" s="8" t="str">
         <f aca="false">IF(A11="","",$B$4&amp;"/"&amp;IF(F11="","en",F11)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A11)&amp;"&amp;utm_source="&amp;IF(E11="","direct",E11)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-2")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=Hypo-Farm&amp;utm_source=whatsapp&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-2</v>
       </c>
       <c r="H11" s="9" t="str">
-        <f aca="false">IF(A11="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F11="ar",$B$7,$B$6),"{name}",IF(B11="","",B11)),"{farm}",A11),"{link}",G11))</f>
-        <v/>
+        <f aca="false">IF(A11="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F11="ar",$B$7,$B$6)," {name}",IF(B11="",""," "&amp;B11)),"{farm}",A11),"{link}",G11))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ Hypo-Farm لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=Hypo-Farm&amp;utm_source=whatsapp&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-2  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I11" s="9" t="str">
         <f aca="false">IF(OR(A11="",D11=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D11,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H11),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J11" s="7"/>
+      <c r="J11" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K11" s="10"/>
-      <c r="L11" s="7"/>
+      <c r="L11" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7"/>
+      <c r="A12" s="7" t="s">
+        <v>35</v>
+      </c>
       <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
+      <c r="C12" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="E12" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G12" s="8" t="str">
         <f aca="false">IF(A12="","",$B$4&amp;"/"&amp;IF(F12="","en",F12)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A12)&amp;"&amp;utm_source="&amp;IF(E12="","direct",E12)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-3")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=Smart%20Green&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-3</v>
       </c>
       <c r="H12" s="9" t="str">
-        <f aca="false">IF(A12="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F12="ar",$B$7,$B$6),"{name}",IF(B12="","",B12)),"{farm}",A12),"{link}",G12))</f>
-        <v/>
+        <f aca="false">IF(A12="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F12="ar",$B$7,$B$6)," {name}",IF(B12="",""," "&amp;B12)),"{farm}",A12),"{link}",G12))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ Smart Green لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=Smart%20Green&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-3  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I12" s="9" t="str">
         <f aca="false">IF(OR(A12="",D12=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D12,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H12),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J12" s="7"/>
+      <c r="J12" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K12" s="10"/>
-      <c r="L12" s="7"/>
+      <c r="L12" s="7" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7"/>
+      <c r="A13" s="7" t="s">
+        <v>37</v>
+      </c>
       <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
+      <c r="C13" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
+      <c r="E13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G13" s="8" t="str">
         <f aca="false">IF(A13="","",$B$4&amp;"/"&amp;IF(F13="","en",F13)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A13)&amp;"&amp;utm_source="&amp;IF(E13="","direct",E13)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-4")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=ECO%20Consult&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-4</v>
       </c>
       <c r="H13" s="9" t="str">
-        <f aca="false">IF(A13="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F13="ar",$B$7,$B$6),"{name}",IF(B13="","",B13)),"{farm}",A13),"{link}",G13))</f>
-        <v/>
+        <f aca="false">IF(A13="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F13="ar",$B$7,$B$6)," {name}",IF(B13="",""," "&amp;B13)),"{farm}",A13),"{link}",G13))</f>
+        <v>Hi, I made a live 3D demo of ECO Consult so you can see how it would look: https://your-domain.com/en/demo?farm=ECO%20Consult&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-4  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I13" s="9" t="str">
         <f aca="false">IF(OR(A13="",D13=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D13,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H13),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J13" s="7"/>
+      <c r="J13" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K13" s="10"/>
-      <c r="L13" s="7"/>
+      <c r="L13" s="7" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7"/>
+      <c r="A14" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
+      <c r="C14" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+      <c r="E14" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G14" s="8" t="str">
         <f aca="false">IF(A14="","",$B$4&amp;"/"&amp;IF(F14="","en",F14)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A14)&amp;"&amp;utm_source="&amp;IF(E14="","direct",E14)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-5")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=HAED-Jo&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-5</v>
       </c>
       <c r="H14" s="9" t="str">
-        <f aca="false">IF(A14="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F14="ar",$B$7,$B$6),"{name}",IF(B14="","",B14)),"{farm}",A14),"{link}",G14))</f>
-        <v/>
+        <f aca="false">IF(A14="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F14="ar",$B$7,$B$6)," {name}",IF(B14="",""," "&amp;B14)),"{farm}",A14),"{link}",G14))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ HAED-Jo لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=HAED-Jo&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-5  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I14" s="9" t="str">
         <f aca="false">IF(OR(A14="",D14=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D14,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H14),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J14" s="7"/>
+      <c r="J14" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K14" s="10"/>
-      <c r="L14" s="7"/>
+      <c r="L14" s="7" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7"/>
+      <c r="A15" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
+      <c r="C15" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
+      <c r="E15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G15" s="8" t="str">
         <f aca="false">IF(A15="","",$B$4&amp;"/"&amp;IF(F15="","en",F15)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A15)&amp;"&amp;utm_source="&amp;IF(E15="","direct",E15)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-6")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=NARC&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-6</v>
       </c>
       <c r="H15" s="9" t="str">
-        <f aca="false">IF(A15="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F15="ar",$B$7,$B$6),"{name}",IF(B15="","",B15)),"{farm}",A15),"{link}",G15))</f>
-        <v/>
+        <f aca="false">IF(A15="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F15="ar",$B$7,$B$6)," {name}",IF(B15="",""," "&amp;B15)),"{farm}",A15),"{link}",G15))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ NARC لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=NARC&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-6  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I15" s="9" t="str">
         <f aca="false">IF(OR(A15="",D15=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D15,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H15),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J15" s="7"/>
+      <c r="J15" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K15" s="10"/>
-      <c r="L15" s="7"/>
+      <c r="L15" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
+      <c r="A16" s="7" t="s">
+        <v>45</v>
+      </c>
       <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
+      <c r="C16" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="E16" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G16" s="8" t="str">
         <f aca="false">IF(A16="","",$B$4&amp;"/"&amp;IF(F16="","en",F16)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A16)&amp;"&amp;utm_source="&amp;IF(E16="","direct",E16)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-7")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=Habak&amp;utm_source=other&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-7</v>
       </c>
       <c r="H16" s="9" t="str">
-        <f aca="false">IF(A16="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F16="ar",$B$7,$B$6),"{name}",IF(B16="","",B16)),"{farm}",A16),"{link}",G16))</f>
-        <v/>
+        <f aca="false">IF(A16="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F16="ar",$B$7,$B$6)," {name}",IF(B16="",""," "&amp;B16)),"{farm}",A16),"{link}",G16))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ Habak لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=Habak&amp;utm_source=other&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-7  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I16" s="9" t="str">
         <f aca="false">IF(OR(A16="",D16=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D16,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H16),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J16" s="7"/>
+      <c r="J16" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K16" s="10"/>
-      <c r="L16" s="7"/>
+      <c r="L16" s="7" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7"/>
+      <c r="A17" s="7" t="s">
+        <v>48</v>
+      </c>
       <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
+      <c r="C17" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
+      <c r="E17" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G17" s="8" t="str">
         <f aca="false">IF(A17="","",$B$4&amp;"/"&amp;IF(F17="","en",F17)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A17)&amp;"&amp;utm_source="&amp;IF(E17="","direct",E17)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-8")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=Badia%20Farms&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-8</v>
       </c>
       <c r="H17" s="9" t="str">
-        <f aca="false">IF(A17="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F17="ar",$B$7,$B$6),"{name}",IF(B17="","",B17)),"{farm}",A17),"{link}",G17))</f>
-        <v/>
+        <f aca="false">IF(A17="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F17="ar",$B$7,$B$6)," {name}",IF(B17="",""," "&amp;B17)),"{farm}",A17),"{link}",G17))</f>
+        <v>Hi, I made a live 3D demo of Badia Farms so you can see how it would look: https://your-domain.com/en/demo?farm=Badia%20Farms&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-8  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I17" s="9" t="str">
         <f aca="false">IF(OR(A17="",D17=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D17,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H17),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J17" s="7"/>
+      <c r="J17" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K17" s="10"/>
-      <c r="L17" s="7"/>
+      <c r="L17" s="7" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
+      <c r="A18" s="7" t="s">
+        <v>51</v>
+      </c>
       <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
+      <c r="C18" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="E18" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G18" s="8" t="str">
         <f aca="false">IF(A18="","",$B$4&amp;"/"&amp;IF(F18="","en",F18)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A18)&amp;"&amp;utm_source="&amp;IF(E18="","direct",E18)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-9")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=Madar%20Farms&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-9</v>
       </c>
       <c r="H18" s="9" t="str">
-        <f aca="false">IF(A18="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F18="ar",$B$7,$B$6),"{name}",IF(B18="","",B18)),"{farm}",A18),"{link}",G18))</f>
-        <v/>
+        <f aca="false">IF(A18="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F18="ar",$B$7,$B$6)," {name}",IF(B18="",""," "&amp;B18)),"{farm}",A18),"{link}",G18))</f>
+        <v>Hi, I made a live 3D demo of Madar Farms so you can see how it would look: https://your-domain.com/en/demo?farm=Madar%20Farms&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-9  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I18" s="9" t="str">
         <f aca="false">IF(OR(A18="",D18=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D18,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H18),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J18" s="7"/>
+      <c r="J18" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K18" s="10"/>
-      <c r="L18" s="7"/>
+      <c r="L18" s="7" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7"/>
+      <c r="A19" s="7" t="s">
+        <v>53</v>
+      </c>
       <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
+      <c r="C19" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
+      <c r="E19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G19" s="8" t="str">
         <f aca="false">IF(A19="","",$B$4&amp;"/"&amp;IF(F19="","en",F19)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A19)&amp;"&amp;utm_source="&amp;IF(E19="","direct",E19)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-10")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=Emirates%20Hydroponics%20Farms&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-10</v>
       </c>
       <c r="H19" s="9" t="str">
-        <f aca="false">IF(A19="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F19="ar",$B$7,$B$6),"{name}",IF(B19="","",B19)),"{farm}",A19),"{link}",G19))</f>
-        <v/>
+        <f aca="false">IF(A19="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F19="ar",$B$7,$B$6)," {name}",IF(B19="",""," "&amp;B19)),"{farm}",A19),"{link}",G19))</f>
+        <v>Hi, I made a live 3D demo of Emirates Hydroponics Farms so you can see how it would look: https://your-domain.com/en/demo?farm=Emirates%20Hydroponics%20Farms&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-10  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I19" s="9" t="str">
         <f aca="false">IF(OR(A19="",D19=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D19,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H19),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J19" s="7"/>
+      <c r="J19" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K19" s="10"/>
-      <c r="L19" s="7"/>
+      <c r="L19" s="7" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7"/>
+      <c r="A20" s="7" t="s">
+        <v>55</v>
+      </c>
       <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
+      <c r="C20" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
+      <c r="E20" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G20" s="8" t="str">
         <f aca="false">IF(A20="","",$B$4&amp;"/"&amp;IF(F20="","en",F20)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A20)&amp;"&amp;utm_source="&amp;IF(E20="","direct",E20)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-11")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=VeggiTech&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-11</v>
       </c>
       <c r="H20" s="9" t="str">
-        <f aca="false">IF(A20="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F20="ar",$B$7,$B$6),"{name}",IF(B20="","",B20)),"{farm}",A20),"{link}",G20))</f>
-        <v/>
+        <f aca="false">IF(A20="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F20="ar",$B$7,$B$6)," {name}",IF(B20="",""," "&amp;B20)),"{farm}",A20),"{link}",G20))</f>
+        <v>Hi, I made a live 3D demo of VeggiTech so you can see how it would look: https://your-domain.com/en/demo?farm=VeggiTech&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-11  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I20" s="9" t="str">
         <f aca="false">IF(OR(A20="",D20=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D20,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H20),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J20" s="7"/>
+      <c r="J20" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K20" s="10"/>
-      <c r="L20" s="7"/>
+      <c r="L20" s="7" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7"/>
+      <c r="A21" s="7" t="s">
+        <v>57</v>
+      </c>
       <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
+      <c r="C21" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
+      <c r="E21" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G21" s="8" t="str">
         <f aca="false">IF(A21="","",$B$4&amp;"/"&amp;IF(F21="","en",F21)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A21)&amp;"&amp;utm_source="&amp;IF(E21="","direct",E21)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-12")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=Emirates%20Bustanica&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-12</v>
       </c>
       <c r="H21" s="9" t="str">
-        <f aca="false">IF(A21="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F21="ar",$B$7,$B$6),"{name}",IF(B21="","",B21)),"{farm}",A21),"{link}",G21))</f>
-        <v/>
+        <f aca="false">IF(A21="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F21="ar",$B$7,$B$6)," {name}",IF(B21="",""," "&amp;B21)),"{farm}",A21),"{link}",G21))</f>
+        <v>Hi, I made a live 3D demo of Emirates Bustanica so you can see how it would look: https://your-domain.com/en/demo?farm=Emirates%20Bustanica&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-12  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I21" s="9" t="str">
         <f aca="false">IF(OR(A21="",D21=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D21,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H21),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J21" s="7"/>
+      <c r="J21" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K21" s="10"/>
-      <c r="L21" s="7"/>
+      <c r="L21" s="7" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7"/>
+      <c r="A22" s="7" t="s">
+        <v>59</v>
+      </c>
       <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
+      <c r="C22" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
+      <c r="E22" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G22" s="8" t="str">
         <f aca="false">IF(A22="","",$B$4&amp;"/"&amp;IF(F22="","en",F22)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A22)&amp;"&amp;utm_source="&amp;IF(E22="","direct",E22)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-13")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=Pure%20Harvest%20Smart%20Farms&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-13</v>
       </c>
       <c r="H22" s="9" t="str">
-        <f aca="false">IF(A22="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F22="ar",$B$7,$B$6),"{name}",IF(B22="","",B22)),"{farm}",A22),"{link}",G22))</f>
-        <v/>
+        <f aca="false">IF(A22="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F22="ar",$B$7,$B$6)," {name}",IF(B22="",""," "&amp;B22)),"{farm}",A22),"{link}",G22))</f>
+        <v>Hi, I made a live 3D demo of Pure Harvest Smart Farms so you can see how it would look: https://your-domain.com/en/demo?farm=Pure%20Harvest%20Smart%20Farms&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-13  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I22" s="9" t="str">
         <f aca="false">IF(OR(A22="",D22=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D22,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H22),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J22" s="7"/>
+      <c r="J22" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K22" s="10"/>
-      <c r="L22" s="7"/>
+      <c r="L22" s="7" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7"/>
+      <c r="A23" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
+      <c r="C23" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
+      <c r="E23" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G23" s="8" t="str">
         <f aca="false">IF(A23="","",$B$4&amp;"/"&amp;IF(F23="","en",F23)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A23)&amp;"&amp;utm_source="&amp;IF(E23="","direct",E23)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-14")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=iFarm&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-14</v>
       </c>
       <c r="H23" s="9" t="str">
-        <f aca="false">IF(A23="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F23="ar",$B$7,$B$6),"{name}",IF(B23="","",B23)),"{farm}",A23),"{link}",G23))</f>
-        <v/>
+        <f aca="false">IF(A23="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F23="ar",$B$7,$B$6)," {name}",IF(B23="",""," "&amp;B23)),"{farm}",A23),"{link}",G23))</f>
+        <v>Hi, I made a live 3D demo of iFarm so you can see how it would look: https://your-domain.com/en/demo?farm=iFarm&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-14  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I23" s="9" t="str">
         <f aca="false">IF(OR(A23="",D23=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D23,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H23),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J23" s="7"/>
+      <c r="J23" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K23" s="10"/>
-      <c r="L23" s="7"/>
+      <c r="L23" s="7" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7"/>
+      <c r="A24" s="7" t="s">
+        <v>63</v>
+      </c>
       <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
+      <c r="C24" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
+      <c r="E24" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G24" s="8" t="str">
         <f aca="false">IF(A24="","",$B$4&amp;"/"&amp;IF(F24="","en",F24)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A24)&amp;"&amp;utm_source="&amp;IF(E24="","direct",E24)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-15")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=ICBA&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-15</v>
       </c>
       <c r="H24" s="9" t="str">
-        <f aca="false">IF(A24="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F24="ar",$B$7,$B$6),"{name}",IF(B24="","",B24)),"{farm}",A24),"{link}",G24))</f>
-        <v/>
+        <f aca="false">IF(A24="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F24="ar",$B$7,$B$6)," {name}",IF(B24="",""," "&amp;B24)),"{farm}",A24),"{link}",G24))</f>
+        <v>Hi, I made a live 3D demo of ICBA so you can see how it would look: https://your-domain.com/en/demo?farm=ICBA&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-15  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I24" s="9" t="str">
         <f aca="false">IF(OR(A24="",D24=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D24,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H24),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J24" s="7"/>
+      <c r="J24" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K24" s="10"/>
-      <c r="L24" s="7"/>
+      <c r="L24" s="7" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7"/>
+      <c r="A25" s="7" t="s">
+        <v>65</v>
+      </c>
       <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
+      <c r="C25" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
+      <c r="E25" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G25" s="8" t="str">
         <f aca="false">IF(A25="","",$B$4&amp;"/"&amp;IF(F25="","en",F25)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A25)&amp;"&amp;utm_source="&amp;IF(E25="","direct",E25)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-16")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=Bather%20Smart%20Farm&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-16</v>
       </c>
       <c r="H25" s="9" t="str">
-        <f aca="false">IF(A25="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F25="ar",$B$7,$B$6),"{name}",IF(B25="","",B25)),"{farm}",A25),"{link}",G25))</f>
-        <v/>
+        <f aca="false">IF(A25="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F25="ar",$B$7,$B$6)," {name}",IF(B25="",""," "&amp;B25)),"{farm}",A25),"{link}",G25))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ Bather Smart Farm لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=Bather%20Smart%20Farm&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-16  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I25" s="9" t="str">
         <f aca="false">IF(OR(A25="",D25=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D25,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H25),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J25" s="7"/>
+      <c r="J25" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K25" s="10"/>
-      <c r="L25" s="7"/>
+      <c r="L25" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7"/>
+      <c r="A26" s="7" t="s">
+        <v>68</v>
+      </c>
       <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
+      <c r="C26" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
+      <c r="E26" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G26" s="8" t="str">
         <f aca="false">IF(A26="","",$B$4&amp;"/"&amp;IF(F26="","en",F26)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A26)&amp;"&amp;utm_source="&amp;IF(E26="","direct",E26)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-17")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=Mojan%20Farms&amp;utm_source=other&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-17</v>
       </c>
       <c r="H26" s="9" t="str">
-        <f aca="false">IF(A26="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F26="ar",$B$7,$B$6),"{name}",IF(B26="","",B26)),"{farm}",A26),"{link}",G26))</f>
-        <v/>
+        <f aca="false">IF(A26="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F26="ar",$B$7,$B$6)," {name}",IF(B26="",""," "&amp;B26)),"{farm}",A26),"{link}",G26))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ Mojan Farms لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=Mojan%20Farms&amp;utm_source=other&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-17  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I26" s="9" t="str">
         <f aca="false">IF(OR(A26="",D26=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D26,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H26),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J26" s="7"/>
+      <c r="J26" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K26" s="10"/>
-      <c r="L26" s="7"/>
+      <c r="L26" s="7" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7"/>
+      <c r="A27" s="7" t="s">
+        <v>70</v>
+      </c>
       <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
+      <c r="C27" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
+      <c r="E27" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G27" s="8" t="str">
         <f aca="false">IF(A27="","",$B$4&amp;"/"&amp;IF(F27="","en",F27)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A27)&amp;"&amp;utm_source="&amp;IF(E27="","direct",E27)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-18")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=Vertical%20Farms%20Company&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-18</v>
       </c>
       <c r="H27" s="9" t="str">
-        <f aca="false">IF(A27="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F27="ar",$B$7,$B$6),"{name}",IF(B27="","",B27)),"{farm}",A27),"{link}",G27))</f>
-        <v/>
+        <f aca="false">IF(A27="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F27="ar",$B$7,$B$6)," {name}",IF(B27="",""," "&amp;B27)),"{farm}",A27),"{link}",G27))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ Vertical Farms Company لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=Vertical%20Farms%20Company&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-18  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I27" s="9" t="str">
         <f aca="false">IF(OR(A27="",D27=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D27,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H27),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J27" s="7"/>
+      <c r="J27" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K27" s="10"/>
-      <c r="L27" s="7"/>
+      <c r="L27" s="7" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7"/>
+      <c r="A28" s="7" t="s">
+        <v>72</v>
+      </c>
       <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
+      <c r="C28" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
+      <c r="E28" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G28" s="8" t="str">
         <f aca="false">IF(A28="","",$B$4&amp;"/"&amp;IF(F28="","en",F28)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A28)&amp;"&amp;utm_source="&amp;IF(E28="","direct",E28)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-19")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=RedSea&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-19</v>
       </c>
       <c r="H28" s="9" t="str">
-        <f aca="false">IF(A28="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F28="ar",$B$7,$B$6),"{name}",IF(B28="","",B28)),"{farm}",A28),"{link}",G28))</f>
-        <v/>
+        <f aca="false">IF(A28="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F28="ar",$B$7,$B$6)," {name}",IF(B28="",""," "&amp;B28)),"{farm}",A28),"{link}",G28))</f>
+        <v>Hi, I made a live 3D demo of RedSea so you can see how it would look: https://your-domain.com/en/demo?farm=RedSea&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-19  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I28" s="9" t="str">
         <f aca="false">IF(OR(A28="",D28=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D28,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H28),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J28" s="7"/>
+      <c r="J28" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K28" s="10"/>
-      <c r="L28" s="7"/>
+      <c r="L28" s="7" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7"/>
+      <c r="A29" s="7" t="s">
+        <v>74</v>
+      </c>
       <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
+      <c r="C29" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
+      <c r="E29" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="G29" s="8" t="str">
         <f aca="false">IF(A29="","",$B$4&amp;"/"&amp;IF(F29="","en",F29)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A29)&amp;"&amp;utm_source="&amp;IF(E29="","direct",E29)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-20")</f>
-        <v/>
+        <v>https://your-domain.com/en/demo?farm=KAUST%20Center%20for%20Desert%20Agriculture&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-20</v>
       </c>
       <c r="H29" s="9" t="str">
-        <f aca="false">IF(A29="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F29="ar",$B$7,$B$6),"{name}",IF(B29="","",B29)),"{farm}",A29),"{link}",G29))</f>
-        <v/>
+        <f aca="false">IF(A29="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F29="ar",$B$7,$B$6)," {name}",IF(B29="",""," "&amp;B29)),"{farm}",A29),"{link}",G29))</f>
+        <v>Hi, I made a live 3D demo of KAUST Center for Desert Agriculture so you can see how it would look: https://your-domain.com/en/demo?farm=KAUST%20Center%20for%20Desert%20Agriculture&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-20  Would you be open to a 30-minute call this week?</v>
       </c>
       <c r="I29" s="9" t="str">
         <f aca="false">IF(OR(A29="",D29=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D29,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H29),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J29" s="7"/>
+      <c r="J29" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K29" s="10"/>
-      <c r="L29" s="7"/>
+      <c r="L29" s="7" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7"/>
+      <c r="A30" s="7" t="s">
+        <v>76</v>
+      </c>
       <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
+      <c r="C30" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
+      <c r="E30" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G30" s="8" t="str">
         <f aca="false">IF(A30="","",$B$4&amp;"/"&amp;IF(F30="","en",F30)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A30)&amp;"&amp;utm_source="&amp;IF(E30="","direct",E30)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-21")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=KACST%20Green%20CEA%20Centre&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-21</v>
       </c>
       <c r="H30" s="9" t="str">
-        <f aca="false">IF(A30="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F30="ar",$B$7,$B$6),"{name}",IF(B30="","",B30)),"{farm}",A30),"{link}",G30))</f>
-        <v/>
+        <f aca="false">IF(A30="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F30="ar",$B$7,$B$6)," {name}",IF(B30="",""," "&amp;B30)),"{farm}",A30),"{link}",G30))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ KACST Green CEA Centre لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=KACST%20Green%20CEA%20Centre&amp;utm_source=email&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-21  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I30" s="9" t="str">
         <f aca="false">IF(OR(A30="",D30=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D30,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H30),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J30" s="7"/>
+      <c r="J30" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K30" s="10"/>
-      <c r="L30" s="7"/>
+      <c r="L30" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7"/>
+      <c r="A31" s="7" t="s">
+        <v>77</v>
+      </c>
       <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
+      <c r="C31" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
+      <c r="E31" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="G31" s="8" t="str">
         <f aca="false">IF(A31="","",$B$4&amp;"/"&amp;IF(F31="","en",F31)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A31)&amp;"&amp;utm_source="&amp;IF(E31="","direct",E31)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-22")</f>
-        <v/>
+        <v>https://your-domain.com/ar/demo?farm=Desert%20Agriculture&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-22</v>
       </c>
       <c r="H31" s="9" t="str">
-        <f aca="false">IF(A31="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F31="ar",$B$7,$B$6),"{name}",IF(B31="","",B31)),"{farm}",A31),"{link}",G31))</f>
-        <v/>
+        <f aca="false">IF(A31="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F31="ar",$B$7,$B$6)," {name}",IF(B31="",""," "&amp;B31)),"{farm}",A31),"{link}",G31))</f>
+        <v>مرحبًا، جهّزت عرضًا حيًّا ثلاثي الأبعاد لـ Desert Agriculture لترى كيف ستبدو مزرعتك: https://your-domain.com/ar/demo?farm=Desert%20Agriculture&amp;utm_source=linkedin&amp;utm_medium=outreach&amp;utm_campaign=outreach-1&amp;utm_content=row-22  هل يناسبك اتصال لمدة 30 دقيقة هذا الأسبوع؟</v>
       </c>
       <c r="I31" s="9" t="str">
         <f aca="false">IF(OR(A31="",D31=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D31,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(H31),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="J31" s="7"/>
+      <c r="J31" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="K31" s="10"/>
-      <c r="L31" s="7"/>
+      <c r="L31" s="7" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7"/>
@@ -1383,7 +1766,7 @@
         <v/>
       </c>
       <c r="H32" s="9" t="str">
-        <f aca="false">IF(A32="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F32="ar",$B$7,$B$6),"{name}",IF(B32="","",B32)),"{farm}",A32),"{link}",G32))</f>
+        <f aca="false">IF(A32="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F32="ar",$B$7,$B$6)," {name}",IF(B32="",""," "&amp;B32)),"{farm}",A32),"{link}",G32))</f>
         <v/>
       </c>
       <c r="I32" s="9" t="str">
@@ -1406,7 +1789,7 @@
         <v/>
       </c>
       <c r="H33" s="9" t="str">
-        <f aca="false">IF(A33="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F33="ar",$B$7,$B$6),"{name}",IF(B33="","",B33)),"{farm}",A33),"{link}",G33))</f>
+        <f aca="false">IF(A33="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F33="ar",$B$7,$B$6)," {name}",IF(B33="",""," "&amp;B33)),"{farm}",A33),"{link}",G33))</f>
         <v/>
       </c>
       <c r="I33" s="9" t="str">
@@ -1429,7 +1812,7 @@
         <v/>
       </c>
       <c r="H34" s="9" t="str">
-        <f aca="false">IF(A34="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F34="ar",$B$7,$B$6),"{name}",IF(B34="","",B34)),"{farm}",A34),"{link}",G34))</f>
+        <f aca="false">IF(A34="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F34="ar",$B$7,$B$6)," {name}",IF(B34="",""," "&amp;B34)),"{farm}",A34),"{link}",G34))</f>
         <v/>
       </c>
       <c r="I34" s="9" t="str">
@@ -1452,7 +1835,7 @@
         <v/>
       </c>
       <c r="H35" s="9" t="str">
-        <f aca="false">IF(A35="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F35="ar",$B$7,$B$6),"{name}",IF(B35="","",B35)),"{farm}",A35),"{link}",G35))</f>
+        <f aca="false">IF(A35="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F35="ar",$B$7,$B$6)," {name}",IF(B35="",""," "&amp;B35)),"{farm}",A35),"{link}",G35))</f>
         <v/>
       </c>
       <c r="I35" s="9" t="str">
@@ -1475,7 +1858,7 @@
         <v/>
       </c>
       <c r="H36" s="9" t="str">
-        <f aca="false">IF(A36="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F36="ar",$B$7,$B$6),"{name}",IF(B36="","",B36)),"{farm}",A36),"{link}",G36))</f>
+        <f aca="false">IF(A36="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F36="ar",$B$7,$B$6)," {name}",IF(B36="",""," "&amp;B36)),"{farm}",A36),"{link}",G36))</f>
         <v/>
       </c>
       <c r="I36" s="9" t="str">
@@ -1498,7 +1881,7 @@
         <v/>
       </c>
       <c r="H37" s="9" t="str">
-        <f aca="false">IF(A37="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F37="ar",$B$7,$B$6),"{name}",IF(B37="","",B37)),"{farm}",A37),"{link}",G37))</f>
+        <f aca="false">IF(A37="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F37="ar",$B$7,$B$6)," {name}",IF(B37="",""," "&amp;B37)),"{farm}",A37),"{link}",G37))</f>
         <v/>
       </c>
       <c r="I37" s="9" t="str">
@@ -1521,7 +1904,7 @@
         <v/>
       </c>
       <c r="H38" s="9" t="str">
-        <f aca="false">IF(A38="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F38="ar",$B$7,$B$6),"{name}",IF(B38="","",B38)),"{farm}",A38),"{link}",G38))</f>
+        <f aca="false">IF(A38="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F38="ar",$B$7,$B$6)," {name}",IF(B38="",""," "&amp;B38)),"{farm}",A38),"{link}",G38))</f>
         <v/>
       </c>
       <c r="I38" s="9" t="str">
@@ -1544,7 +1927,7 @@
         <v/>
       </c>
       <c r="H39" s="9" t="str">
-        <f aca="false">IF(A39="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F39="ar",$B$7,$B$6),"{name}",IF(B39="","",B39)),"{farm}",A39),"{link}",G39))</f>
+        <f aca="false">IF(A39="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F39="ar",$B$7,$B$6)," {name}",IF(B39="",""," "&amp;B39)),"{farm}",A39),"{link}",G39))</f>
         <v/>
       </c>
       <c r="I39" s="9" t="str">
@@ -1567,7 +1950,7 @@
         <v/>
       </c>
       <c r="H40" s="9" t="str">
-        <f aca="false">IF(A40="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F40="ar",$B$7,$B$6),"{name}",IF(B40="","",B40)),"{farm}",A40),"{link}",G40))</f>
+        <f aca="false">IF(A40="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F40="ar",$B$7,$B$6)," {name}",IF(B40="",""," "&amp;B40)),"{farm}",A40),"{link}",G40))</f>
         <v/>
       </c>
       <c r="I40" s="9" t="str">
@@ -1590,7 +1973,7 @@
         <v/>
       </c>
       <c r="H41" s="9" t="str">
-        <f aca="false">IF(A41="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F41="ar",$B$7,$B$6),"{name}",IF(B41="","",B41)),"{farm}",A41),"{link}",G41))</f>
+        <f aca="false">IF(A41="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F41="ar",$B$7,$B$6)," {name}",IF(B41="",""," "&amp;B41)),"{farm}",A41),"{link}",G41))</f>
         <v/>
       </c>
       <c r="I41" s="9" t="str">
@@ -1613,7 +1996,7 @@
         <v/>
       </c>
       <c r="H42" s="9" t="str">
-        <f aca="false">IF(A42="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F42="ar",$B$7,$B$6),"{name}",IF(B42="","",B42)),"{farm}",A42),"{link}",G42))</f>
+        <f aca="false">IF(A42="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F42="ar",$B$7,$B$6)," {name}",IF(B42="",""," "&amp;B42)),"{farm}",A42),"{link}",G42))</f>
         <v/>
       </c>
       <c r="I42" s="9" t="str">
@@ -1636,7 +2019,7 @@
         <v/>
       </c>
       <c r="H43" s="9" t="str">
-        <f aca="false">IF(A43="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F43="ar",$B$7,$B$6),"{name}",IF(B43="","",B43)),"{farm}",A43),"{link}",G43))</f>
+        <f aca="false">IF(A43="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F43="ar",$B$7,$B$6)," {name}",IF(B43="",""," "&amp;B43)),"{farm}",A43),"{link}",G43))</f>
         <v/>
       </c>
       <c r="I43" s="9" t="str">
@@ -1659,7 +2042,7 @@
         <v/>
       </c>
       <c r="H44" s="9" t="str">
-        <f aca="false">IF(A44="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F44="ar",$B$7,$B$6),"{name}",IF(B44="","",B44)),"{farm}",A44),"{link}",G44))</f>
+        <f aca="false">IF(A44="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F44="ar",$B$7,$B$6)," {name}",IF(B44="",""," "&amp;B44)),"{farm}",A44),"{link}",G44))</f>
         <v/>
       </c>
       <c r="I44" s="9" t="str">
@@ -1682,7 +2065,7 @@
         <v/>
       </c>
       <c r="H45" s="9" t="str">
-        <f aca="false">IF(A45="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F45="ar",$B$7,$B$6),"{name}",IF(B45="","",B45)),"{farm}",A45),"{link}",G45))</f>
+        <f aca="false">IF(A45="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F45="ar",$B$7,$B$6)," {name}",IF(B45="",""," "&amp;B45)),"{farm}",A45),"{link}",G45))</f>
         <v/>
       </c>
       <c r="I45" s="9" t="str">
@@ -1705,7 +2088,7 @@
         <v/>
       </c>
       <c r="H46" s="9" t="str">
-        <f aca="false">IF(A46="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F46="ar",$B$7,$B$6),"{name}",IF(B46="","",B46)),"{farm}",A46),"{link}",G46))</f>
+        <f aca="false">IF(A46="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F46="ar",$B$7,$B$6)," {name}",IF(B46="",""," "&amp;B46)),"{farm}",A46),"{link}",G46))</f>
         <v/>
       </c>
       <c r="I46" s="9" t="str">
@@ -1728,7 +2111,7 @@
         <v/>
       </c>
       <c r="H47" s="9" t="str">
-        <f aca="false">IF(A47="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F47="ar",$B$7,$B$6),"{name}",IF(B47="","",B47)),"{farm}",A47),"{link}",G47))</f>
+        <f aca="false">IF(A47="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F47="ar",$B$7,$B$6)," {name}",IF(B47="",""," "&amp;B47)),"{farm}",A47),"{link}",G47))</f>
         <v/>
       </c>
       <c r="I47" s="9" t="str">
@@ -1751,7 +2134,7 @@
         <v/>
       </c>
       <c r="H48" s="9" t="str">
-        <f aca="false">IF(A48="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F48="ar",$B$7,$B$6),"{name}",IF(B48="","",B48)),"{farm}",A48),"{link}",G48))</f>
+        <f aca="false">IF(A48="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F48="ar",$B$7,$B$6)," {name}",IF(B48="",""," "&amp;B48)),"{farm}",A48),"{link}",G48))</f>
         <v/>
       </c>
       <c r="I48" s="9" t="str">
@@ -1774,7 +2157,7 @@
         <v/>
       </c>
       <c r="H49" s="9" t="str">
-        <f aca="false">IF(A49="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F49="ar",$B$7,$B$6),"{name}",IF(B49="","",B49)),"{farm}",A49),"{link}",G49))</f>
+        <f aca="false">IF(A49="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F49="ar",$B$7,$B$6)," {name}",IF(B49="",""," "&amp;B49)),"{farm}",A49),"{link}",G49))</f>
         <v/>
       </c>
       <c r="I49" s="9" t="str">
@@ -1797,7 +2180,7 @@
         <v/>
       </c>
       <c r="H50" s="9" t="str">
-        <f aca="false">IF(A50="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F50="ar",$B$7,$B$6),"{name}",IF(B50="","",B50)),"{farm}",A50),"{link}",G50))</f>
+        <f aca="false">IF(A50="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F50="ar",$B$7,$B$6)," {name}",IF(B50="",""," "&amp;B50)),"{farm}",A50),"{link}",G50))</f>
         <v/>
       </c>
       <c r="I50" s="9" t="str">
@@ -1820,7 +2203,7 @@
         <v/>
       </c>
       <c r="H51" s="9" t="str">
-        <f aca="false">IF(A51="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F51="ar",$B$7,$B$6),"{name}",IF(B51="","",B51)),"{farm}",A51),"{link}",G51))</f>
+        <f aca="false">IF(A51="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F51="ar",$B$7,$B$6)," {name}",IF(B51="",""," "&amp;B51)),"{farm}",A51),"{link}",G51))</f>
         <v/>
       </c>
       <c r="I51" s="9" t="str">
@@ -1843,7 +2226,7 @@
         <v/>
       </c>
       <c r="H52" s="9" t="str">
-        <f aca="false">IF(A52="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F52="ar",$B$7,$B$6),"{name}",IF(B52="","",B52)),"{farm}",A52),"{link}",G52))</f>
+        <f aca="false">IF(A52="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F52="ar",$B$7,$B$6)," {name}",IF(B52="",""," "&amp;B52)),"{farm}",A52),"{link}",G52))</f>
         <v/>
       </c>
       <c r="I52" s="9" t="str">
@@ -1866,7 +2249,7 @@
         <v/>
       </c>
       <c r="H53" s="9" t="str">
-        <f aca="false">IF(A53="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F53="ar",$B$7,$B$6),"{name}",IF(B53="","",B53)),"{farm}",A53),"{link}",G53))</f>
+        <f aca="false">IF(A53="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F53="ar",$B$7,$B$6)," {name}",IF(B53="",""," "&amp;B53)),"{farm}",A53),"{link}",G53))</f>
         <v/>
       </c>
       <c r="I53" s="9" t="str">
@@ -1889,7 +2272,7 @@
         <v/>
       </c>
       <c r="H54" s="9" t="str">
-        <f aca="false">IF(A54="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F54="ar",$B$7,$B$6),"{name}",IF(B54="","",B54)),"{farm}",A54),"{link}",G54))</f>
+        <f aca="false">IF(A54="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F54="ar",$B$7,$B$6)," {name}",IF(B54="",""," "&amp;B54)),"{farm}",A54),"{link}",G54))</f>
         <v/>
       </c>
       <c r="I54" s="9" t="str">
@@ -1912,7 +2295,7 @@
         <v/>
       </c>
       <c r="H55" s="9" t="str">
-        <f aca="false">IF(A55="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F55="ar",$B$7,$B$6),"{name}",IF(B55="","",B55)),"{farm}",A55),"{link}",G55))</f>
+        <f aca="false">IF(A55="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F55="ar",$B$7,$B$6)," {name}",IF(B55="",""," "&amp;B55)),"{farm}",A55),"{link}",G55))</f>
         <v/>
       </c>
       <c r="I55" s="9" t="str">
@@ -1935,7 +2318,7 @@
         <v/>
       </c>
       <c r="H56" s="9" t="str">
-        <f aca="false">IF(A56="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F56="ar",$B$7,$B$6),"{name}",IF(B56="","",B56)),"{farm}",A56),"{link}",G56))</f>
+        <f aca="false">IF(A56="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F56="ar",$B$7,$B$6)," {name}",IF(B56="",""," "&amp;B56)),"{farm}",A56),"{link}",G56))</f>
         <v/>
       </c>
       <c r="I56" s="9" t="str">
@@ -1958,7 +2341,7 @@
         <v/>
       </c>
       <c r="H57" s="9" t="str">
-        <f aca="false">IF(A57="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F57="ar",$B$7,$B$6),"{name}",IF(B57="","",B57)),"{farm}",A57),"{link}",G57))</f>
+        <f aca="false">IF(A57="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F57="ar",$B$7,$B$6)," {name}",IF(B57="",""," "&amp;B57)),"{farm}",A57),"{link}",G57))</f>
         <v/>
       </c>
       <c r="I57" s="9" t="str">
@@ -1981,7 +2364,7 @@
         <v/>
       </c>
       <c r="H58" s="9" t="str">
-        <f aca="false">IF(A58="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F58="ar",$B$7,$B$6),"{name}",IF(B58="","",B58)),"{farm}",A58),"{link}",G58))</f>
+        <f aca="false">IF(A58="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F58="ar",$B$7,$B$6)," {name}",IF(B58="",""," "&amp;B58)),"{farm}",A58),"{link}",G58))</f>
         <v/>
       </c>
       <c r="I58" s="9" t="str">
@@ -2004,7 +2387,7 @@
         <v/>
       </c>
       <c r="H59" s="9" t="str">
-        <f aca="false">IF(A59="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F59="ar",$B$7,$B$6),"{name}",IF(B59="","",B59)),"{farm}",A59),"{link}",G59))</f>
+        <f aca="false">IF(A59="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F59="ar",$B$7,$B$6)," {name}",IF(B59="",""," "&amp;B59)),"{farm}",A59),"{link}",G59))</f>
         <v/>
       </c>
       <c r="I59" s="9" t="str">
@@ -2027,7 +2410,7 @@
         <v/>
       </c>
       <c r="H60" s="9" t="str">
-        <f aca="false">IF(A60="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F60="ar",$B$7,$B$6),"{name}",IF(B60="","",B60)),"{farm}",A60),"{link}",G60))</f>
+        <f aca="false">IF(A60="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F60="ar",$B$7,$B$6)," {name}",IF(B60="",""," "&amp;B60)),"{farm}",A60),"{link}",G60))</f>
         <v/>
       </c>
       <c r="I60" s="9" t="str">
@@ -2050,7 +2433,7 @@
         <v/>
       </c>
       <c r="H61" s="9" t="str">
-        <f aca="false">IF(A61="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F61="ar",$B$7,$B$6),"{name}",IF(B61="","",B61)),"{farm}",A61),"{link}",G61))</f>
+        <f aca="false">IF(A61="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F61="ar",$B$7,$B$6)," {name}",IF(B61="",""," "&amp;B61)),"{farm}",A61),"{link}",G61))</f>
         <v/>
       </c>
       <c r="I61" s="9" t="str">
@@ -2073,7 +2456,7 @@
         <v/>
       </c>
       <c r="H62" s="9" t="str">
-        <f aca="false">IF(A62="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F62="ar",$B$7,$B$6),"{name}",IF(B62="","",B62)),"{farm}",A62),"{link}",G62))</f>
+        <f aca="false">IF(A62="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F62="ar",$B$7,$B$6)," {name}",IF(B62="",""," "&amp;B62)),"{farm}",A62),"{link}",G62))</f>
         <v/>
       </c>
       <c r="I62" s="9" t="str">
@@ -2096,7 +2479,7 @@
         <v/>
       </c>
       <c r="H63" s="9" t="str">
-        <f aca="false">IF(A63="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F63="ar",$B$7,$B$6),"{name}",IF(B63="","",B63)),"{farm}",A63),"{link}",G63))</f>
+        <f aca="false">IF(A63="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F63="ar",$B$7,$B$6)," {name}",IF(B63="",""," "&amp;B63)),"{farm}",A63),"{link}",G63))</f>
         <v/>
       </c>
       <c r="I63" s="9" t="str">
@@ -2119,7 +2502,7 @@
         <v/>
       </c>
       <c r="H64" s="9" t="str">
-        <f aca="false">IF(A64="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F64="ar",$B$7,$B$6),"{name}",IF(B64="","",B64)),"{farm}",A64),"{link}",G64))</f>
+        <f aca="false">IF(A64="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F64="ar",$B$7,$B$6)," {name}",IF(B64="",""," "&amp;B64)),"{farm}",A64),"{link}",G64))</f>
         <v/>
       </c>
       <c r="I64" s="9" t="str">
@@ -2142,7 +2525,7 @@
         <v/>
       </c>
       <c r="H65" s="9" t="str">
-        <f aca="false">IF(A65="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F65="ar",$B$7,$B$6),"{name}",IF(B65="","",B65)),"{farm}",A65),"{link}",G65))</f>
+        <f aca="false">IF(A65="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F65="ar",$B$7,$B$6)," {name}",IF(B65="",""," "&amp;B65)),"{farm}",A65),"{link}",G65))</f>
         <v/>
       </c>
       <c r="I65" s="9" t="str">
@@ -2165,7 +2548,7 @@
         <v/>
       </c>
       <c r="H66" s="9" t="str">
-        <f aca="false">IF(A66="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F66="ar",$B$7,$B$6),"{name}",IF(B66="","",B66)),"{farm}",A66),"{link}",G66))</f>
+        <f aca="false">IF(A66="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F66="ar",$B$7,$B$6)," {name}",IF(B66="",""," "&amp;B66)),"{farm}",A66),"{link}",G66))</f>
         <v/>
       </c>
       <c r="I66" s="9" t="str">
@@ -2188,7 +2571,7 @@
         <v/>
       </c>
       <c r="H67" s="9" t="str">
-        <f aca="false">IF(A67="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F67="ar",$B$7,$B$6),"{name}",IF(B67="","",B67)),"{farm}",A67),"{link}",G67))</f>
+        <f aca="false">IF(A67="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F67="ar",$B$7,$B$6)," {name}",IF(B67="",""," "&amp;B67)),"{farm}",A67),"{link}",G67))</f>
         <v/>
       </c>
       <c r="I67" s="9" t="str">
@@ -2211,7 +2594,7 @@
         <v/>
       </c>
       <c r="H68" s="9" t="str">
-        <f aca="false">IF(A68="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F68="ar",$B$7,$B$6),"{name}",IF(B68="","",B68)),"{farm}",A68),"{link}",G68))</f>
+        <f aca="false">IF(A68="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F68="ar",$B$7,$B$6)," {name}",IF(B68="",""," "&amp;B68)),"{farm}",A68),"{link}",G68))</f>
         <v/>
       </c>
       <c r="I68" s="9" t="str">
@@ -2234,7 +2617,7 @@
         <v/>
       </c>
       <c r="H69" s="9" t="str">
-        <f aca="false">IF(A69="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F69="ar",$B$7,$B$6),"{name}",IF(B69="","",B69)),"{farm}",A69),"{link}",G69))</f>
+        <f aca="false">IF(A69="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F69="ar",$B$7,$B$6)," {name}",IF(B69="",""," "&amp;B69)),"{farm}",A69),"{link}",G69))</f>
         <v/>
       </c>
       <c r="I69" s="9" t="str">
@@ -2257,7 +2640,7 @@
         <v/>
       </c>
       <c r="H70" s="9" t="str">
-        <f aca="false">IF(A70="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F70="ar",$B$7,$B$6),"{name}",IF(B70="","",B70)),"{farm}",A70),"{link}",G70))</f>
+        <f aca="false">IF(A70="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F70="ar",$B$7,$B$6)," {name}",IF(B70="",""," "&amp;B70)),"{farm}",A70),"{link}",G70))</f>
         <v/>
       </c>
       <c r="I70" s="9" t="str">
@@ -2280,7 +2663,7 @@
         <v/>
       </c>
       <c r="H71" s="9" t="str">
-        <f aca="false">IF(A71="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F71="ar",$B$7,$B$6),"{name}",IF(B71="","",B71)),"{farm}",A71),"{link}",G71))</f>
+        <f aca="false">IF(A71="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F71="ar",$B$7,$B$6)," {name}",IF(B71="",""," "&amp;B71)),"{farm}",A71),"{link}",G71))</f>
         <v/>
       </c>
       <c r="I71" s="9" t="str">
@@ -2303,7 +2686,7 @@
         <v/>
       </c>
       <c r="H72" s="9" t="str">
-        <f aca="false">IF(A72="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F72="ar",$B$7,$B$6),"{name}",IF(B72="","",B72)),"{farm}",A72),"{link}",G72))</f>
+        <f aca="false">IF(A72="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F72="ar",$B$7,$B$6)," {name}",IF(B72="",""," "&amp;B72)),"{farm}",A72),"{link}",G72))</f>
         <v/>
       </c>
       <c r="I72" s="9" t="str">
@@ -2326,7 +2709,7 @@
         <v/>
       </c>
       <c r="H73" s="9" t="str">
-        <f aca="false">IF(A73="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F73="ar",$B$7,$B$6),"{name}",IF(B73="","",B73)),"{farm}",A73),"{link}",G73))</f>
+        <f aca="false">IF(A73="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F73="ar",$B$7,$B$6)," {name}",IF(B73="",""," "&amp;B73)),"{farm}",A73),"{link}",G73))</f>
         <v/>
       </c>
       <c r="I73" s="9" t="str">
@@ -2349,7 +2732,7 @@
         <v/>
       </c>
       <c r="H74" s="9" t="str">
-        <f aca="false">IF(A74="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F74="ar",$B$7,$B$6),"{name}",IF(B74="","",B74)),"{farm}",A74),"{link}",G74))</f>
+        <f aca="false">IF(A74="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F74="ar",$B$7,$B$6)," {name}",IF(B74="",""," "&amp;B74)),"{farm}",A74),"{link}",G74))</f>
         <v/>
       </c>
       <c r="I74" s="9" t="str">
@@ -2372,7 +2755,7 @@
         <v/>
       </c>
       <c r="H75" s="9" t="str">
-        <f aca="false">IF(A75="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F75="ar",$B$7,$B$6),"{name}",IF(B75="","",B75)),"{farm}",A75),"{link}",G75))</f>
+        <f aca="false">IF(A75="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F75="ar",$B$7,$B$6)," {name}",IF(B75="",""," "&amp;B75)),"{farm}",A75),"{link}",G75))</f>
         <v/>
       </c>
       <c r="I75" s="9" t="str">
@@ -2395,7 +2778,7 @@
         <v/>
       </c>
       <c r="H76" s="9" t="str">
-        <f aca="false">IF(A76="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F76="ar",$B$7,$B$6),"{name}",IF(B76="","",B76)),"{farm}",A76),"{link}",G76))</f>
+        <f aca="false">IF(A76="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F76="ar",$B$7,$B$6)," {name}",IF(B76="",""," "&amp;B76)),"{farm}",A76),"{link}",G76))</f>
         <v/>
       </c>
       <c r="I76" s="9" t="str">
@@ -2418,7 +2801,7 @@
         <v/>
       </c>
       <c r="H77" s="9" t="str">
-        <f aca="false">IF(A77="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F77="ar",$B$7,$B$6),"{name}",IF(B77="","",B77)),"{farm}",A77),"{link}",G77))</f>
+        <f aca="false">IF(A77="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F77="ar",$B$7,$B$6)," {name}",IF(B77="",""," "&amp;B77)),"{farm}",A77),"{link}",G77))</f>
         <v/>
       </c>
       <c r="I77" s="9" t="str">
@@ -2441,7 +2824,7 @@
         <v/>
       </c>
       <c r="H78" s="9" t="str">
-        <f aca="false">IF(A78="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F78="ar",$B$7,$B$6),"{name}",IF(B78="","",B78)),"{farm}",A78),"{link}",G78))</f>
+        <f aca="false">IF(A78="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F78="ar",$B$7,$B$6)," {name}",IF(B78="",""," "&amp;B78)),"{farm}",A78),"{link}",G78))</f>
         <v/>
       </c>
       <c r="I78" s="9" t="str">
@@ -2464,7 +2847,7 @@
         <v/>
       </c>
       <c r="H79" s="9" t="str">
-        <f aca="false">IF(A79="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F79="ar",$B$7,$B$6),"{name}",IF(B79="","",B79)),"{farm}",A79),"{link}",G79))</f>
+        <f aca="false">IF(A79="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F79="ar",$B$7,$B$6)," {name}",IF(B79="",""," "&amp;B79)),"{farm}",A79),"{link}",G79))</f>
         <v/>
       </c>
       <c r="I79" s="9" t="str">
@@ -2487,7 +2870,7 @@
         <v/>
       </c>
       <c r="H80" s="9" t="str">
-        <f aca="false">IF(A80="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F80="ar",$B$7,$B$6),"{name}",IF(B80="","",B80)),"{farm}",A80),"{link}",G80))</f>
+        <f aca="false">IF(A80="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F80="ar",$B$7,$B$6)," {name}",IF(B80="",""," "&amp;B80)),"{farm}",A80),"{link}",G80))</f>
         <v/>
       </c>
       <c r="I80" s="9" t="str">
@@ -2510,7 +2893,7 @@
         <v/>
       </c>
       <c r="H81" s="9" t="str">
-        <f aca="false">IF(A81="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F81="ar",$B$7,$B$6),"{name}",IF(B81="","",B81)),"{farm}",A81),"{link}",G81))</f>
+        <f aca="false">IF(A81="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F81="ar",$B$7,$B$6)," {name}",IF(B81="",""," "&amp;B81)),"{farm}",A81),"{link}",G81))</f>
         <v/>
       </c>
       <c r="I81" s="9" t="str">
@@ -2533,7 +2916,7 @@
         <v/>
       </c>
       <c r="H82" s="9" t="str">
-        <f aca="false">IF(A82="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F82="ar",$B$7,$B$6),"{name}",IF(B82="","",B82)),"{farm}",A82),"{link}",G82))</f>
+        <f aca="false">IF(A82="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F82="ar",$B$7,$B$6)," {name}",IF(B82="",""," "&amp;B82)),"{farm}",A82),"{link}",G82))</f>
         <v/>
       </c>
       <c r="I82" s="9" t="str">
@@ -2556,7 +2939,7 @@
         <v/>
       </c>
       <c r="H83" s="9" t="str">
-        <f aca="false">IF(A83="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F83="ar",$B$7,$B$6),"{name}",IF(B83="","",B83)),"{farm}",A83),"{link}",G83))</f>
+        <f aca="false">IF(A83="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F83="ar",$B$7,$B$6)," {name}",IF(B83="",""," "&amp;B83)),"{farm}",A83),"{link}",G83))</f>
         <v/>
       </c>
       <c r="I83" s="9" t="str">
@@ -2579,7 +2962,7 @@
         <v/>
       </c>
       <c r="H84" s="9" t="str">
-        <f aca="false">IF(A84="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F84="ar",$B$7,$B$6),"{name}",IF(B84="","",B84)),"{farm}",A84),"{link}",G84))</f>
+        <f aca="false">IF(A84="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F84="ar",$B$7,$B$6)," {name}",IF(B84="",""," "&amp;B84)),"{farm}",A84),"{link}",G84))</f>
         <v/>
       </c>
       <c r="I84" s="9" t="str">
@@ -2602,7 +2985,7 @@
         <v/>
       </c>
       <c r="H85" s="9" t="str">
-        <f aca="false">IF(A85="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F85="ar",$B$7,$B$6),"{name}",IF(B85="","",B85)),"{farm}",A85),"{link}",G85))</f>
+        <f aca="false">IF(A85="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F85="ar",$B$7,$B$6)," {name}",IF(B85="",""," "&amp;B85)),"{farm}",A85),"{link}",G85))</f>
         <v/>
       </c>
       <c r="I85" s="9" t="str">
@@ -2625,7 +3008,7 @@
         <v/>
       </c>
       <c r="H86" s="9" t="str">
-        <f aca="false">IF(A86="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F86="ar",$B$7,$B$6),"{name}",IF(B86="","",B86)),"{farm}",A86),"{link}",G86))</f>
+        <f aca="false">IF(A86="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F86="ar",$B$7,$B$6)," {name}",IF(B86="",""," "&amp;B86)),"{farm}",A86),"{link}",G86))</f>
         <v/>
       </c>
       <c r="I86" s="9" t="str">
@@ -2648,7 +3031,7 @@
         <v/>
       </c>
       <c r="H87" s="9" t="str">
-        <f aca="false">IF(A87="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F87="ar",$B$7,$B$6),"{name}",IF(B87="","",B87)),"{farm}",A87),"{link}",G87))</f>
+        <f aca="false">IF(A87="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F87="ar",$B$7,$B$6)," {name}",IF(B87="",""," "&amp;B87)),"{farm}",A87),"{link}",G87))</f>
         <v/>
       </c>
       <c r="I87" s="9" t="str">
@@ -2671,7 +3054,7 @@
         <v/>
       </c>
       <c r="H88" s="9" t="str">
-        <f aca="false">IF(A88="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F88="ar",$B$7,$B$6),"{name}",IF(B88="","",B88)),"{farm}",A88),"{link}",G88))</f>
+        <f aca="false">IF(A88="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F88="ar",$B$7,$B$6)," {name}",IF(B88="",""," "&amp;B88)),"{farm}",A88),"{link}",G88))</f>
         <v/>
       </c>
       <c r="I88" s="9" t="str">
@@ -2694,7 +3077,7 @@
         <v/>
       </c>
       <c r="H89" s="9" t="str">
-        <f aca="false">IF(A89="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F89="ar",$B$7,$B$6),"{name}",IF(B89="","",B89)),"{farm}",A89),"{link}",G89))</f>
+        <f aca="false">IF(A89="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F89="ar",$B$7,$B$6)," {name}",IF(B89="",""," "&amp;B89)),"{farm}",A89),"{link}",G89))</f>
         <v/>
       </c>
       <c r="I89" s="9" t="str">
@@ -2717,7 +3100,7 @@
         <v/>
       </c>
       <c r="H90" s="9" t="str">
-        <f aca="false">IF(A90="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F90="ar",$B$7,$B$6),"{name}",IF(B90="","",B90)),"{farm}",A90),"{link}",G90))</f>
+        <f aca="false">IF(A90="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F90="ar",$B$7,$B$6)," {name}",IF(B90="",""," "&amp;B90)),"{farm}",A90),"{link}",G90))</f>
         <v/>
       </c>
       <c r="I90" s="9" t="str">
@@ -2740,7 +3123,7 @@
         <v/>
       </c>
       <c r="H91" s="9" t="str">
-        <f aca="false">IF(A91="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F91="ar",$B$7,$B$6),"{name}",IF(B91="","",B91)),"{farm}",A91),"{link}",G91))</f>
+        <f aca="false">IF(A91="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F91="ar",$B$7,$B$6)," {name}",IF(B91="",""," "&amp;B91)),"{farm}",A91),"{link}",G91))</f>
         <v/>
       </c>
       <c r="I91" s="9" t="str">
@@ -2763,7 +3146,7 @@
         <v/>
       </c>
       <c r="H92" s="9" t="str">
-        <f aca="false">IF(A92="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F92="ar",$B$7,$B$6),"{name}",IF(B92="","",B92)),"{farm}",A92),"{link}",G92))</f>
+        <f aca="false">IF(A92="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F92="ar",$B$7,$B$6)," {name}",IF(B92="",""," "&amp;B92)),"{farm}",A92),"{link}",G92))</f>
         <v/>
       </c>
       <c r="I92" s="9" t="str">
@@ -2786,7 +3169,7 @@
         <v/>
       </c>
       <c r="H93" s="9" t="str">
-        <f aca="false">IF(A93="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F93="ar",$B$7,$B$6),"{name}",IF(B93="","",B93)),"{farm}",A93),"{link}",G93))</f>
+        <f aca="false">IF(A93="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F93="ar",$B$7,$B$6)," {name}",IF(B93="",""," "&amp;B93)),"{farm}",A93),"{link}",G93))</f>
         <v/>
       </c>
       <c r="I93" s="9" t="str">
@@ -2809,7 +3192,7 @@
         <v/>
       </c>
       <c r="H94" s="9" t="str">
-        <f aca="false">IF(A94="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F94="ar",$B$7,$B$6),"{name}",IF(B94="","",B94)),"{farm}",A94),"{link}",G94))</f>
+        <f aca="false">IF(A94="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F94="ar",$B$7,$B$6)," {name}",IF(B94="",""," "&amp;B94)),"{farm}",A94),"{link}",G94))</f>
         <v/>
       </c>
       <c r="I94" s="9" t="str">
@@ -2832,7 +3215,7 @@
         <v/>
       </c>
       <c r="H95" s="9" t="str">
-        <f aca="false">IF(A95="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F95="ar",$B$7,$B$6),"{name}",IF(B95="","",B95)),"{farm}",A95),"{link}",G95))</f>
+        <f aca="false">IF(A95="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F95="ar",$B$7,$B$6)," {name}",IF(B95="",""," "&amp;B95)),"{farm}",A95),"{link}",G95))</f>
         <v/>
       </c>
       <c r="I95" s="9" t="str">
@@ -2855,7 +3238,7 @@
         <v/>
       </c>
       <c r="H96" s="9" t="str">
-        <f aca="false">IF(A96="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F96="ar",$B$7,$B$6),"{name}",IF(B96="","",B96)),"{farm}",A96),"{link}",G96))</f>
+        <f aca="false">IF(A96="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F96="ar",$B$7,$B$6)," {name}",IF(B96="",""," "&amp;B96)),"{farm}",A96),"{link}",G96))</f>
         <v/>
       </c>
       <c r="I96" s="9" t="str">
@@ -2878,7 +3261,7 @@
         <v/>
       </c>
       <c r="H97" s="9" t="str">
-        <f aca="false">IF(A97="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F97="ar",$B$7,$B$6),"{name}",IF(B97="","",B97)),"{farm}",A97),"{link}",G97))</f>
+        <f aca="false">IF(A97="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F97="ar",$B$7,$B$6)," {name}",IF(B97="",""," "&amp;B97)),"{farm}",A97),"{link}",G97))</f>
         <v/>
       </c>
       <c r="I97" s="9" t="str">
@@ -2901,7 +3284,7 @@
         <v/>
       </c>
       <c r="H98" s="9" t="str">
-        <f aca="false">IF(A98="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F98="ar",$B$7,$B$6),"{name}",IF(B98="","",B98)),"{farm}",A98),"{link}",G98))</f>
+        <f aca="false">IF(A98="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F98="ar",$B$7,$B$6)," {name}",IF(B98="",""," "&amp;B98)),"{farm}",A98),"{link}",G98))</f>
         <v/>
       </c>
       <c r="I98" s="9" t="str">
@@ -2924,7 +3307,7 @@
         <v/>
       </c>
       <c r="H99" s="9" t="str">
-        <f aca="false">IF(A99="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F99="ar",$B$7,$B$6),"{name}",IF(B99="","",B99)),"{farm}",A99),"{link}",G99))</f>
+        <f aca="false">IF(A99="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F99="ar",$B$7,$B$6)," {name}",IF(B99="",""," "&amp;B99)),"{farm}",A99),"{link}",G99))</f>
         <v/>
       </c>
       <c r="I99" s="9" t="str">
@@ -2947,7 +3330,7 @@
         <v/>
       </c>
       <c r="H100" s="9" t="str">
-        <f aca="false">IF(A100="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F100="ar",$B$7,$B$6),"{name}",IF(B100="","",B100)),"{farm}",A100),"{link}",G100))</f>
+        <f aca="false">IF(A100="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F100="ar",$B$7,$B$6)," {name}",IF(B100="",""," "&amp;B100)),"{farm}",A100),"{link}",G100))</f>
         <v/>
       </c>
       <c r="I100" s="9" t="str">
@@ -2970,7 +3353,7 @@
         <v/>
       </c>
       <c r="H101" s="9" t="str">
-        <f aca="false">IF(A101="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F101="ar",$B$7,$B$6),"{name}",IF(B101="","",B101)),"{farm}",A101),"{link}",G101))</f>
+        <f aca="false">IF(A101="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F101="ar",$B$7,$B$6)," {name}",IF(B101="",""," "&amp;B101)),"{farm}",A101),"{link}",G101))</f>
         <v/>
       </c>
       <c r="I101" s="9" t="str">
@@ -2993,7 +3376,7 @@
         <v/>
       </c>
       <c r="H102" s="9" t="str">
-        <f aca="false">IF(A102="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F102="ar",$B$7,$B$6),"{name}",IF(B102="","",B102)),"{farm}",A102),"{link}",G102))</f>
+        <f aca="false">IF(A102="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F102="ar",$B$7,$B$6)," {name}",IF(B102="",""," "&amp;B102)),"{farm}",A102),"{link}",G102))</f>
         <v/>
       </c>
       <c r="I102" s="9" t="str">
@@ -3016,7 +3399,7 @@
         <v/>
       </c>
       <c r="H103" s="9" t="str">
-        <f aca="false">IF(A103="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F103="ar",$B$7,$B$6),"{name}",IF(B103="","",B103)),"{farm}",A103),"{link}",G103))</f>
+        <f aca="false">IF(A103="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F103="ar",$B$7,$B$6)," {name}",IF(B103="",""," "&amp;B103)),"{farm}",A103),"{link}",G103))</f>
         <v/>
       </c>
       <c r="I103" s="9" t="str">
@@ -3039,7 +3422,7 @@
         <v/>
       </c>
       <c r="H104" s="9" t="str">
-        <f aca="false">IF(A104="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F104="ar",$B$7,$B$6),"{name}",IF(B104="","",B104)),"{farm}",A104),"{link}",G104))</f>
+        <f aca="false">IF(A104="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F104="ar",$B$7,$B$6)," {name}",IF(B104="",""," "&amp;B104)),"{farm}",A104),"{link}",G104))</f>
         <v/>
       </c>
       <c r="I104" s="9" t="str">
@@ -3062,7 +3445,7 @@
         <v/>
       </c>
       <c r="H105" s="9" t="str">
-        <f aca="false">IF(A105="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F105="ar",$B$7,$B$6),"{name}",IF(B105="","",B105)),"{farm}",A105),"{link}",G105))</f>
+        <f aca="false">IF(A105="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F105="ar",$B$7,$B$6)," {name}",IF(B105="",""," "&amp;B105)),"{farm}",A105),"{link}",G105))</f>
         <v/>
       </c>
       <c r="I105" s="9" t="str">
@@ -3085,7 +3468,7 @@
         <v/>
       </c>
       <c r="H106" s="9" t="str">
-        <f aca="false">IF(A106="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F106="ar",$B$7,$B$6),"{name}",IF(B106="","",B106)),"{farm}",A106),"{link}",G106))</f>
+        <f aca="false">IF(A106="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F106="ar",$B$7,$B$6)," {name}",IF(B106="",""," "&amp;B106)),"{farm}",A106),"{link}",G106))</f>
         <v/>
       </c>
       <c r="I106" s="9" t="str">
@@ -3108,7 +3491,7 @@
         <v/>
       </c>
       <c r="H107" s="9" t="str">
-        <f aca="false">IF(A107="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F107="ar",$B$7,$B$6),"{name}",IF(B107="","",B107)),"{farm}",A107),"{link}",G107))</f>
+        <f aca="false">IF(A107="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F107="ar",$B$7,$B$6)," {name}",IF(B107="",""," "&amp;B107)),"{farm}",A107),"{link}",G107))</f>
         <v/>
       </c>
       <c r="I107" s="9" t="str">
@@ -3131,7 +3514,7 @@
         <v/>
       </c>
       <c r="H108" s="9" t="str">
-        <f aca="false">IF(A108="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F108="ar",$B$7,$B$6),"{name}",IF(B108="","",B108)),"{farm}",A108),"{link}",G108))</f>
+        <f aca="false">IF(A108="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F108="ar",$B$7,$B$6)," {name}",IF(B108="",""," "&amp;B108)),"{farm}",A108),"{link}",G108))</f>
         <v/>
       </c>
       <c r="I108" s="9" t="str">
@@ -3154,7 +3537,7 @@
         <v/>
       </c>
       <c r="H109" s="9" t="str">
-        <f aca="false">IF(A109="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F109="ar",$B$7,$B$6),"{name}",IF(B109="","",B109)),"{farm}",A109),"{link}",G109))</f>
+        <f aca="false">IF(A109="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F109="ar",$B$7,$B$6)," {name}",IF(B109="",""," "&amp;B109)),"{farm}",A109),"{link}",G109))</f>
         <v/>
       </c>
       <c r="I109" s="9" t="str">
@@ -3177,7 +3560,7 @@
         <v/>
       </c>
       <c r="H110" s="9" t="str">
-        <f aca="false">IF(A110="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F110="ar",$B$7,$B$6),"{name}",IF(B110="","",B110)),"{farm}",A110),"{link}",G110))</f>
+        <f aca="false">IF(A110="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F110="ar",$B$7,$B$6)," {name}",IF(B110="",""," "&amp;B110)),"{farm}",A110),"{link}",G110))</f>
         <v/>
       </c>
       <c r="I110" s="9" t="str">
@@ -3200,7 +3583,7 @@
         <v/>
       </c>
       <c r="H111" s="9" t="str">
-        <f aca="false">IF(A111="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F111="ar",$B$7,$B$6),"{name}",IF(B111="","",B111)),"{farm}",A111),"{link}",G111))</f>
+        <f aca="false">IF(A111="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F111="ar",$B$7,$B$6)," {name}",IF(B111="",""," "&amp;B111)),"{farm}",A111),"{link}",G111))</f>
         <v/>
       </c>
       <c r="I111" s="9" t="str">
@@ -3223,7 +3606,7 @@
         <v/>
       </c>
       <c r="H112" s="9" t="str">
-        <f aca="false">IF(A112="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F112="ar",$B$7,$B$6),"{name}",IF(B112="","",B112)),"{farm}",A112),"{link}",G112))</f>
+        <f aca="false">IF(A112="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F112="ar",$B$7,$B$6)," {name}",IF(B112="",""," "&amp;B112)),"{farm}",A112),"{link}",G112))</f>
         <v/>
       </c>
       <c r="I112" s="9" t="str">
@@ -3246,7 +3629,7 @@
         <v/>
       </c>
       <c r="H113" s="9" t="str">
-        <f aca="false">IF(A113="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F113="ar",$B$7,$B$6),"{name}",IF(B113="","",B113)),"{farm}",A113),"{link}",G113))</f>
+        <f aca="false">IF(A113="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F113="ar",$B$7,$B$6)," {name}",IF(B113="",""," "&amp;B113)),"{farm}",A113),"{link}",G113))</f>
         <v/>
       </c>
       <c r="I113" s="9" t="str">
@@ -3269,7 +3652,7 @@
         <v/>
       </c>
       <c r="H114" s="9" t="str">
-        <f aca="false">IF(A114="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F114="ar",$B$7,$B$6),"{name}",IF(B114="","",B114)),"{farm}",A114),"{link}",G114))</f>
+        <f aca="false">IF(A114="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F114="ar",$B$7,$B$6)," {name}",IF(B114="",""," "&amp;B114)),"{farm}",A114),"{link}",G114))</f>
         <v/>
       </c>
       <c r="I114" s="9" t="str">
@@ -3292,7 +3675,7 @@
         <v/>
       </c>
       <c r="H115" s="9" t="str">
-        <f aca="false">IF(A115="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F115="ar",$B$7,$B$6),"{name}",IF(B115="","",B115)),"{farm}",A115),"{link}",G115))</f>
+        <f aca="false">IF(A115="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F115="ar",$B$7,$B$6)," {name}",IF(B115="",""," "&amp;B115)),"{farm}",A115),"{link}",G115))</f>
         <v/>
       </c>
       <c r="I115" s="9" t="str">
@@ -3315,7 +3698,7 @@
         <v/>
       </c>
       <c r="H116" s="9" t="str">
-        <f aca="false">IF(A116="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F116="ar",$B$7,$B$6),"{name}",IF(B116="","",B116)),"{farm}",A116),"{link}",G116))</f>
+        <f aca="false">IF(A116="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F116="ar",$B$7,$B$6)," {name}",IF(B116="",""," "&amp;B116)),"{farm}",A116),"{link}",G116))</f>
         <v/>
       </c>
       <c r="I116" s="9" t="str">
@@ -3338,7 +3721,7 @@
         <v/>
       </c>
       <c r="H117" s="9" t="str">
-        <f aca="false">IF(A117="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F117="ar",$B$7,$B$6),"{name}",IF(B117="","",B117)),"{farm}",A117),"{link}",G117))</f>
+        <f aca="false">IF(A117="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F117="ar",$B$7,$B$6)," {name}",IF(B117="",""," "&amp;B117)),"{farm}",A117),"{link}",G117))</f>
         <v/>
       </c>
       <c r="I117" s="9" t="str">
@@ -3361,7 +3744,7 @@
         <v/>
       </c>
       <c r="H118" s="9" t="str">
-        <f aca="false">IF(A118="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F118="ar",$B$7,$B$6),"{name}",IF(B118="","",B118)),"{farm}",A118),"{link}",G118))</f>
+        <f aca="false">IF(A118="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F118="ar",$B$7,$B$6)," {name}",IF(B118="",""," "&amp;B118)),"{farm}",A118),"{link}",G118))</f>
         <v/>
       </c>
       <c r="I118" s="9" t="str">
@@ -3384,7 +3767,7 @@
         <v/>
       </c>
       <c r="H119" s="9" t="str">
-        <f aca="false">IF(A119="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F119="ar",$B$7,$B$6),"{name}",IF(B119="","",B119)),"{farm}",A119),"{link}",G119))</f>
+        <f aca="false">IF(A119="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F119="ar",$B$7,$B$6)," {name}",IF(B119="",""," "&amp;B119)),"{farm}",A119),"{link}",G119))</f>
         <v/>
       </c>
       <c r="I119" s="9" t="str">
@@ -3407,7 +3790,7 @@
         <v/>
       </c>
       <c r="H120" s="9" t="str">
-        <f aca="false">IF(A120="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F120="ar",$B$7,$B$6),"{name}",IF(B120="","",B120)),"{farm}",A120),"{link}",G120))</f>
+        <f aca="false">IF(A120="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F120="ar",$B$7,$B$6)," {name}",IF(B120="",""," "&amp;B120)),"{farm}",A120),"{link}",G120))</f>
         <v/>
       </c>
       <c r="I120" s="9" t="str">
@@ -3430,7 +3813,7 @@
         <v/>
       </c>
       <c r="H121" s="9" t="str">
-        <f aca="false">IF(A121="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F121="ar",$B$7,$B$6),"{name}",IF(B121="","",B121)),"{farm}",A121),"{link}",G121))</f>
+        <f aca="false">IF(A121="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F121="ar",$B$7,$B$6)," {name}",IF(B121="",""," "&amp;B121)),"{farm}",A121),"{link}",G121))</f>
         <v/>
       </c>
       <c r="I121" s="9" t="str">
@@ -3453,7 +3836,7 @@
         <v/>
       </c>
       <c r="H122" s="9" t="str">
-        <f aca="false">IF(A122="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F122="ar",$B$7,$B$6),"{name}",IF(B122="","",B122)),"{farm}",A122),"{link}",G122))</f>
+        <f aca="false">IF(A122="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F122="ar",$B$7,$B$6)," {name}",IF(B122="",""," "&amp;B122)),"{farm}",A122),"{link}",G122))</f>
         <v/>
       </c>
       <c r="I122" s="9" t="str">
@@ -3476,7 +3859,7 @@
         <v/>
       </c>
       <c r="H123" s="9" t="str">
-        <f aca="false">IF(A123="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F123="ar",$B$7,$B$6),"{name}",IF(B123="","",B123)),"{farm}",A123),"{link}",G123))</f>
+        <f aca="false">IF(A123="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F123="ar",$B$7,$B$6)," {name}",IF(B123="",""," "&amp;B123)),"{farm}",A123),"{link}",G123))</f>
         <v/>
       </c>
       <c r="I123" s="9" t="str">
@@ -3499,7 +3882,7 @@
         <v/>
       </c>
       <c r="H124" s="9" t="str">
-        <f aca="false">IF(A124="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F124="ar",$B$7,$B$6),"{name}",IF(B124="","",B124)),"{farm}",A124),"{link}",G124))</f>
+        <f aca="false">IF(A124="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F124="ar",$B$7,$B$6)," {name}",IF(B124="",""," "&amp;B124)),"{farm}",A124),"{link}",G124))</f>
         <v/>
       </c>
       <c r="I124" s="9" t="str">
@@ -3522,7 +3905,7 @@
         <v/>
       </c>
       <c r="H125" s="9" t="str">
-        <f aca="false">IF(A125="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F125="ar",$B$7,$B$6),"{name}",IF(B125="","",B125)),"{farm}",A125),"{link}",G125))</f>
+        <f aca="false">IF(A125="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F125="ar",$B$7,$B$6)," {name}",IF(B125="",""," "&amp;B125)),"{farm}",A125),"{link}",G125))</f>
         <v/>
       </c>
       <c r="I125" s="9" t="str">
@@ -3545,7 +3928,7 @@
         <v/>
       </c>
       <c r="H126" s="9" t="str">
-        <f aca="false">IF(A126="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F126="ar",$B$7,$B$6),"{name}",IF(B126="","",B126)),"{farm}",A126),"{link}",G126))</f>
+        <f aca="false">IF(A126="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F126="ar",$B$7,$B$6)," {name}",IF(B126="",""," "&amp;B126)),"{farm}",A126),"{link}",G126))</f>
         <v/>
       </c>
       <c r="I126" s="9" t="str">
@@ -3568,7 +3951,7 @@
         <v/>
       </c>
       <c r="H127" s="9" t="str">
-        <f aca="false">IF(A127="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F127="ar",$B$7,$B$6),"{name}",IF(B127="","",B127)),"{farm}",A127),"{link}",G127))</f>
+        <f aca="false">IF(A127="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F127="ar",$B$7,$B$6)," {name}",IF(B127="",""," "&amp;B127)),"{farm}",A127),"{link}",G127))</f>
         <v/>
       </c>
       <c r="I127" s="9" t="str">
@@ -3591,7 +3974,7 @@
         <v/>
       </c>
       <c r="H128" s="9" t="str">
-        <f aca="false">IF(A128="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F128="ar",$B$7,$B$6),"{name}",IF(B128="","",B128)),"{farm}",A128),"{link}",G128))</f>
+        <f aca="false">IF(A128="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F128="ar",$B$7,$B$6)," {name}",IF(B128="",""," "&amp;B128)),"{farm}",A128),"{link}",G128))</f>
         <v/>
       </c>
       <c r="I128" s="9" t="str">
@@ -3614,7 +3997,7 @@
         <v/>
       </c>
       <c r="H129" s="9" t="str">
-        <f aca="false">IF(A129="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F129="ar",$B$7,$B$6),"{name}",IF(B129="","",B129)),"{farm}",A129),"{link}",G129))</f>
+        <f aca="false">IF(A129="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F129="ar",$B$7,$B$6)," {name}",IF(B129="",""," "&amp;B129)),"{farm}",A129),"{link}",G129))</f>
         <v/>
       </c>
       <c r="I129" s="9" t="str">
@@ -3637,7 +4020,7 @@
         <v/>
       </c>
       <c r="H130" s="9" t="str">
-        <f aca="false">IF(A130="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F130="ar",$B$7,$B$6),"{name}",IF(B130="","",B130)),"{farm}",A130),"{link}",G130))</f>
+        <f aca="false">IF(A130="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F130="ar",$B$7,$B$6)," {name}",IF(B130="",""," "&amp;B130)),"{farm}",A130),"{link}",G130))</f>
         <v/>
       </c>
       <c r="I130" s="9" t="str">
@@ -3660,7 +4043,7 @@
         <v/>
       </c>
       <c r="H131" s="9" t="str">
-        <f aca="false">IF(A131="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F131="ar",$B$7,$B$6),"{name}",IF(B131="","",B131)),"{farm}",A131),"{link}",G131))</f>
+        <f aca="false">IF(A131="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F131="ar",$B$7,$B$6)," {name}",IF(B131="",""," "&amp;B131)),"{farm}",A131),"{link}",G131))</f>
         <v/>
       </c>
       <c r="I131" s="9" t="str">
@@ -3683,7 +4066,7 @@
         <v/>
       </c>
       <c r="H132" s="9" t="str">
-        <f aca="false">IF(A132="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F132="ar",$B$7,$B$6),"{name}",IF(B132="","",B132)),"{farm}",A132),"{link}",G132))</f>
+        <f aca="false">IF(A132="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F132="ar",$B$7,$B$6)," {name}",IF(B132="",""," "&amp;B132)),"{farm}",A132),"{link}",G132))</f>
         <v/>
       </c>
       <c r="I132" s="9" t="str">
@@ -3706,7 +4089,7 @@
         <v/>
       </c>
       <c r="H133" s="9" t="str">
-        <f aca="false">IF(A133="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F133="ar",$B$7,$B$6),"{name}",IF(B133="","",B133)),"{farm}",A133),"{link}",G133))</f>
+        <f aca="false">IF(A133="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F133="ar",$B$7,$B$6)," {name}",IF(B133="",""," "&amp;B133)),"{farm}",A133),"{link}",G133))</f>
         <v/>
       </c>
       <c r="I133" s="9" t="str">
@@ -3729,7 +4112,7 @@
         <v/>
       </c>
       <c r="H134" s="9" t="str">
-        <f aca="false">IF(A134="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F134="ar",$B$7,$B$6),"{name}",IF(B134="","",B134)),"{farm}",A134),"{link}",G134))</f>
+        <f aca="false">IF(A134="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F134="ar",$B$7,$B$6)," {name}",IF(B134="",""," "&amp;B134)),"{farm}",A134),"{link}",G134))</f>
         <v/>
       </c>
       <c r="I134" s="9" t="str">
@@ -3752,7 +4135,7 @@
         <v/>
       </c>
       <c r="H135" s="9" t="str">
-        <f aca="false">IF(A135="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F135="ar",$B$7,$B$6),"{name}",IF(B135="","",B135)),"{farm}",A135),"{link}",G135))</f>
+        <f aca="false">IF(A135="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F135="ar",$B$7,$B$6)," {name}",IF(B135="",""," "&amp;B135)),"{farm}",A135),"{link}",G135))</f>
         <v/>
       </c>
       <c r="I135" s="9" t="str">
@@ -3775,7 +4158,7 @@
         <v/>
       </c>
       <c r="H136" s="9" t="str">
-        <f aca="false">IF(A136="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F136="ar",$B$7,$B$6),"{name}",IF(B136="","",B136)),"{farm}",A136),"{link}",G136))</f>
+        <f aca="false">IF(A136="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F136="ar",$B$7,$B$6)," {name}",IF(B136="",""," "&amp;B136)),"{farm}",A136),"{link}",G136))</f>
         <v/>
       </c>
       <c r="I136" s="9" t="str">
@@ -3798,7 +4181,7 @@
         <v/>
       </c>
       <c r="H137" s="9" t="str">
-        <f aca="false">IF(A137="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F137="ar",$B$7,$B$6),"{name}",IF(B137="","",B137)),"{farm}",A137),"{link}",G137))</f>
+        <f aca="false">IF(A137="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F137="ar",$B$7,$B$6)," {name}",IF(B137="",""," "&amp;B137)),"{farm}",A137),"{link}",G137))</f>
         <v/>
       </c>
       <c r="I137" s="9" t="str">
@@ -3821,7 +4204,7 @@
         <v/>
       </c>
       <c r="H138" s="9" t="str">
-        <f aca="false">IF(A138="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F138="ar",$B$7,$B$6),"{name}",IF(B138="","",B138)),"{farm}",A138),"{link}",G138))</f>
+        <f aca="false">IF(A138="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F138="ar",$B$7,$B$6)," {name}",IF(B138="",""," "&amp;B138)),"{farm}",A138),"{link}",G138))</f>
         <v/>
       </c>
       <c r="I138" s="9" t="str">
@@ -3844,7 +4227,7 @@
         <v/>
       </c>
       <c r="H139" s="9" t="str">
-        <f aca="false">IF(A139="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F139="ar",$B$7,$B$6),"{name}",IF(B139="","",B139)),"{farm}",A139),"{link}",G139))</f>
+        <f aca="false">IF(A139="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F139="ar",$B$7,$B$6)," {name}",IF(B139="",""," "&amp;B139)),"{farm}",A139),"{link}",G139))</f>
         <v/>
       </c>
       <c r="I139" s="9" t="str">
@@ -3867,7 +4250,7 @@
         <v/>
       </c>
       <c r="H140" s="9" t="str">
-        <f aca="false">IF(A140="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F140="ar",$B$7,$B$6),"{name}",IF(B140="","",B140)),"{farm}",A140),"{link}",G140))</f>
+        <f aca="false">IF(A140="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F140="ar",$B$7,$B$6)," {name}",IF(B140="",""," "&amp;B140)),"{farm}",A140),"{link}",G140))</f>
         <v/>
       </c>
       <c r="I140" s="9" t="str">
@@ -3890,7 +4273,7 @@
         <v/>
       </c>
       <c r="H141" s="9" t="str">
-        <f aca="false">IF(A141="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F141="ar",$B$7,$B$6),"{name}",IF(B141="","",B141)),"{farm}",A141),"{link}",G141))</f>
+        <f aca="false">IF(A141="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F141="ar",$B$7,$B$6)," {name}",IF(B141="",""," "&amp;B141)),"{farm}",A141),"{link}",G141))</f>
         <v/>
       </c>
       <c r="I141" s="9" t="str">
@@ -3913,7 +4296,7 @@
         <v/>
       </c>
       <c r="H142" s="9" t="str">
-        <f aca="false">IF(A142="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F142="ar",$B$7,$B$6),"{name}",IF(B142="","",B142)),"{farm}",A142),"{link}",G142))</f>
+        <f aca="false">IF(A142="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F142="ar",$B$7,$B$6)," {name}",IF(B142="",""," "&amp;B142)),"{farm}",A142),"{link}",G142))</f>
         <v/>
       </c>
       <c r="I142" s="9" t="str">
@@ -3936,7 +4319,7 @@
         <v/>
       </c>
       <c r="H143" s="9" t="str">
-        <f aca="false">IF(A143="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F143="ar",$B$7,$B$6),"{name}",IF(B143="","",B143)),"{farm}",A143),"{link}",G143))</f>
+        <f aca="false">IF(A143="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F143="ar",$B$7,$B$6)," {name}",IF(B143="",""," "&amp;B143)),"{farm}",A143),"{link}",G143))</f>
         <v/>
       </c>
       <c r="I143" s="9" t="str">
@@ -3959,7 +4342,7 @@
         <v/>
       </c>
       <c r="H144" s="9" t="str">
-        <f aca="false">IF(A144="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F144="ar",$B$7,$B$6),"{name}",IF(B144="","",B144)),"{farm}",A144),"{link}",G144))</f>
+        <f aca="false">IF(A144="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F144="ar",$B$7,$B$6)," {name}",IF(B144="",""," "&amp;B144)),"{farm}",A144),"{link}",G144))</f>
         <v/>
       </c>
       <c r="I144" s="9" t="str">
@@ -3982,7 +4365,7 @@
         <v/>
       </c>
       <c r="H145" s="9" t="str">
-        <f aca="false">IF(A145="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F145="ar",$B$7,$B$6),"{name}",IF(B145="","",B145)),"{farm}",A145),"{link}",G145))</f>
+        <f aca="false">IF(A145="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F145="ar",$B$7,$B$6)," {name}",IF(B145="",""," "&amp;B145)),"{farm}",A145),"{link}",G145))</f>
         <v/>
       </c>
       <c r="I145" s="9" t="str">
@@ -4005,7 +4388,7 @@
         <v/>
       </c>
       <c r="H146" s="9" t="str">
-        <f aca="false">IF(A146="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F146="ar",$B$7,$B$6),"{name}",IF(B146="","",B146)),"{farm}",A146),"{link}",G146))</f>
+        <f aca="false">IF(A146="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F146="ar",$B$7,$B$6)," {name}",IF(B146="",""," "&amp;B146)),"{farm}",A146),"{link}",G146))</f>
         <v/>
       </c>
       <c r="I146" s="9" t="str">
@@ -4028,7 +4411,7 @@
         <v/>
       </c>
       <c r="H147" s="9" t="str">
-        <f aca="false">IF(A147="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F147="ar",$B$7,$B$6),"{name}",IF(B147="","",B147)),"{farm}",A147),"{link}",G147))</f>
+        <f aca="false">IF(A147="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F147="ar",$B$7,$B$6)," {name}",IF(B147="",""," "&amp;B147)),"{farm}",A147),"{link}",G147))</f>
         <v/>
       </c>
       <c r="I147" s="9" t="str">
@@ -4051,7 +4434,7 @@
         <v/>
       </c>
       <c r="H148" s="9" t="str">
-        <f aca="false">IF(A148="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F148="ar",$B$7,$B$6),"{name}",IF(B148="","",B148)),"{farm}",A148),"{link}",G148))</f>
+        <f aca="false">IF(A148="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F148="ar",$B$7,$B$6)," {name}",IF(B148="",""," "&amp;B148)),"{farm}",A148),"{link}",G148))</f>
         <v/>
       </c>
       <c r="I148" s="9" t="str">
@@ -4074,7 +4457,7 @@
         <v/>
       </c>
       <c r="H149" s="9" t="str">
-        <f aca="false">IF(A149="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F149="ar",$B$7,$B$6),"{name}",IF(B149="","",B149)),"{farm}",A149),"{link}",G149))</f>
+        <f aca="false">IF(A149="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F149="ar",$B$7,$B$6)," {name}",IF(B149="",""," "&amp;B149)),"{farm}",A149),"{link}",G149))</f>
         <v/>
       </c>
       <c r="I149" s="9" t="str">
@@ -4097,7 +4480,7 @@
         <v/>
       </c>
       <c r="H150" s="9" t="str">
-        <f aca="false">IF(A150="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F150="ar",$B$7,$B$6),"{name}",IF(B150="","",B150)),"{farm}",A150),"{link}",G150))</f>
+        <f aca="false">IF(A150="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F150="ar",$B$7,$B$6)," {name}",IF(B150="",""," "&amp;B150)),"{farm}",A150),"{link}",G150))</f>
         <v/>
       </c>
       <c r="I150" s="9" t="str">
@@ -4120,7 +4503,7 @@
         <v/>
       </c>
       <c r="H151" s="9" t="str">
-        <f aca="false">IF(A151="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F151="ar",$B$7,$B$6),"{name}",IF(B151="","",B151)),"{farm}",A151),"{link}",G151))</f>
+        <f aca="false">IF(A151="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F151="ar",$B$7,$B$6)," {name}",IF(B151="",""," "&amp;B151)),"{farm}",A151),"{link}",G151))</f>
         <v/>
       </c>
       <c r="I151" s="9" t="str">
@@ -4143,7 +4526,7 @@
         <v/>
       </c>
       <c r="H152" s="9" t="str">
-        <f aca="false">IF(A152="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F152="ar",$B$7,$B$6),"{name}",IF(B152="","",B152)),"{farm}",A152),"{link}",G152))</f>
+        <f aca="false">IF(A152="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F152="ar",$B$7,$B$6)," {name}",IF(B152="",""," "&amp;B152)),"{farm}",A152),"{link}",G152))</f>
         <v/>
       </c>
       <c r="I152" s="9" t="str">
@@ -4166,7 +4549,7 @@
         <v/>
       </c>
       <c r="H153" s="9" t="str">
-        <f aca="false">IF(A153="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F153="ar",$B$7,$B$6),"{name}",IF(B153="","",B153)),"{farm}",A153),"{link}",G153))</f>
+        <f aca="false">IF(A153="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F153="ar",$B$7,$B$6)," {name}",IF(B153="",""," "&amp;B153)),"{farm}",A153),"{link}",G153))</f>
         <v/>
       </c>
       <c r="I153" s="9" t="str">
@@ -4189,7 +4572,7 @@
         <v/>
       </c>
       <c r="H154" s="9" t="str">
-        <f aca="false">IF(A154="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F154="ar",$B$7,$B$6),"{name}",IF(B154="","",B154)),"{farm}",A154),"{link}",G154))</f>
+        <f aca="false">IF(A154="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F154="ar",$B$7,$B$6)," {name}",IF(B154="",""," "&amp;B154)),"{farm}",A154),"{link}",G154))</f>
         <v/>
       </c>
       <c r="I154" s="9" t="str">
@@ -4212,7 +4595,7 @@
         <v/>
       </c>
       <c r="H155" s="9" t="str">
-        <f aca="false">IF(A155="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F155="ar",$B$7,$B$6),"{name}",IF(B155="","",B155)),"{farm}",A155),"{link}",G155))</f>
+        <f aca="false">IF(A155="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F155="ar",$B$7,$B$6)," {name}",IF(B155="",""," "&amp;B155)),"{farm}",A155),"{link}",G155))</f>
         <v/>
       </c>
       <c r="I155" s="9" t="str">
@@ -4235,7 +4618,7 @@
         <v/>
       </c>
       <c r="H156" s="9" t="str">
-        <f aca="false">IF(A156="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F156="ar",$B$7,$B$6),"{name}",IF(B156="","",B156)),"{farm}",A156),"{link}",G156))</f>
+        <f aca="false">IF(A156="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F156="ar",$B$7,$B$6)," {name}",IF(B156="",""," "&amp;B156)),"{farm}",A156),"{link}",G156))</f>
         <v/>
       </c>
       <c r="I156" s="9" t="str">
@@ -4258,7 +4641,7 @@
         <v/>
       </c>
       <c r="H157" s="9" t="str">
-        <f aca="false">IF(A157="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F157="ar",$B$7,$B$6),"{name}",IF(B157="","",B157)),"{farm}",A157),"{link}",G157))</f>
+        <f aca="false">IF(A157="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F157="ar",$B$7,$B$6)," {name}",IF(B157="",""," "&amp;B157)),"{farm}",A157),"{link}",G157))</f>
         <v/>
       </c>
       <c r="I157" s="9" t="str">
@@ -4281,7 +4664,7 @@
         <v/>
       </c>
       <c r="H158" s="9" t="str">
-        <f aca="false">IF(A158="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F158="ar",$B$7,$B$6),"{name}",IF(B158="","",B158)),"{farm}",A158),"{link}",G158))</f>
+        <f aca="false">IF(A158="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F158="ar",$B$7,$B$6)," {name}",IF(B158="",""," "&amp;B158)),"{farm}",A158),"{link}",G158))</f>
         <v/>
       </c>
       <c r="I158" s="9" t="str">
@@ -4304,7 +4687,7 @@
         <v/>
       </c>
       <c r="H159" s="9" t="str">
-        <f aca="false">IF(A159="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F159="ar",$B$7,$B$6),"{name}",IF(B159="","",B159)),"{farm}",A159),"{link}",G159))</f>
+        <f aca="false">IF(A159="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F159="ar",$B$7,$B$6)," {name}",IF(B159="",""," "&amp;B159)),"{farm}",A159),"{link}",G159))</f>
         <v/>
       </c>
       <c r="I159" s="9" t="str">
@@ -4327,7 +4710,7 @@
         <v/>
       </c>
       <c r="H160" s="9" t="str">
-        <f aca="false">IF(A160="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F160="ar",$B$7,$B$6),"{name}",IF(B160="","",B160)),"{farm}",A160),"{link}",G160))</f>
+        <f aca="false">IF(A160="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F160="ar",$B$7,$B$6)," {name}",IF(B160="",""," "&amp;B160)),"{farm}",A160),"{link}",G160))</f>
         <v/>
       </c>
       <c r="I160" s="9" t="str">
@@ -4350,7 +4733,7 @@
         <v/>
       </c>
       <c r="H161" s="9" t="str">
-        <f aca="false">IF(A161="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F161="ar",$B$7,$B$6),"{name}",IF(B161="","",B161)),"{farm}",A161),"{link}",G161))</f>
+        <f aca="false">IF(A161="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F161="ar",$B$7,$B$6)," {name}",IF(B161="",""," "&amp;B161)),"{farm}",A161),"{link}",G161))</f>
         <v/>
       </c>
       <c r="I161" s="9" t="str">
@@ -4373,7 +4756,7 @@
         <v/>
       </c>
       <c r="H162" s="9" t="str">
-        <f aca="false">IF(A162="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F162="ar",$B$7,$B$6),"{name}",IF(B162="","",B162)),"{farm}",A162),"{link}",G162))</f>
+        <f aca="false">IF(A162="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F162="ar",$B$7,$B$6)," {name}",IF(B162="",""," "&amp;B162)),"{farm}",A162),"{link}",G162))</f>
         <v/>
       </c>
       <c r="I162" s="9" t="str">
@@ -4396,7 +4779,7 @@
         <v/>
       </c>
       <c r="H163" s="9" t="str">
-        <f aca="false">IF(A163="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F163="ar",$B$7,$B$6),"{name}",IF(B163="","",B163)),"{farm}",A163),"{link}",G163))</f>
+        <f aca="false">IF(A163="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F163="ar",$B$7,$B$6)," {name}",IF(B163="",""," "&amp;B163)),"{farm}",A163),"{link}",G163))</f>
         <v/>
       </c>
       <c r="I163" s="9" t="str">
@@ -4419,7 +4802,7 @@
         <v/>
       </c>
       <c r="H164" s="9" t="str">
-        <f aca="false">IF(A164="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F164="ar",$B$7,$B$6),"{name}",IF(B164="","",B164)),"{farm}",A164),"{link}",G164))</f>
+        <f aca="false">IF(A164="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F164="ar",$B$7,$B$6)," {name}",IF(B164="",""," "&amp;B164)),"{farm}",A164),"{link}",G164))</f>
         <v/>
       </c>
       <c r="I164" s="9" t="str">
@@ -4442,7 +4825,7 @@
         <v/>
       </c>
       <c r="H165" s="9" t="str">
-        <f aca="false">IF(A165="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F165="ar",$B$7,$B$6),"{name}",IF(B165="","",B165)),"{farm}",A165),"{link}",G165))</f>
+        <f aca="false">IF(A165="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F165="ar",$B$7,$B$6)," {name}",IF(B165="",""," "&amp;B165)),"{farm}",A165),"{link}",G165))</f>
         <v/>
       </c>
       <c r="I165" s="9" t="str">
@@ -4465,7 +4848,7 @@
         <v/>
       </c>
       <c r="H166" s="9" t="str">
-        <f aca="false">IF(A166="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F166="ar",$B$7,$B$6),"{name}",IF(B166="","",B166)),"{farm}",A166),"{link}",G166))</f>
+        <f aca="false">IF(A166="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F166="ar",$B$7,$B$6)," {name}",IF(B166="",""," "&amp;B166)),"{farm}",A166),"{link}",G166))</f>
         <v/>
       </c>
       <c r="I166" s="9" t="str">
@@ -4488,7 +4871,7 @@
         <v/>
       </c>
       <c r="H167" s="9" t="str">
-        <f aca="false">IF(A167="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F167="ar",$B$7,$B$6),"{name}",IF(B167="","",B167)),"{farm}",A167),"{link}",G167))</f>
+        <f aca="false">IF(A167="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F167="ar",$B$7,$B$6)," {name}",IF(B167="",""," "&amp;B167)),"{farm}",A167),"{link}",G167))</f>
         <v/>
       </c>
       <c r="I167" s="9" t="str">
@@ -4511,7 +4894,7 @@
         <v/>
       </c>
       <c r="H168" s="9" t="str">
-        <f aca="false">IF(A168="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F168="ar",$B$7,$B$6),"{name}",IF(B168="","",B168)),"{farm}",A168),"{link}",G168))</f>
+        <f aca="false">IF(A168="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F168="ar",$B$7,$B$6)," {name}",IF(B168="",""," "&amp;B168)),"{farm}",A168),"{link}",G168))</f>
         <v/>
       </c>
       <c r="I168" s="9" t="str">
@@ -4534,7 +4917,7 @@
         <v/>
       </c>
       <c r="H169" s="9" t="str">
-        <f aca="false">IF(A169="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F169="ar",$B$7,$B$6),"{name}",IF(B169="","",B169)),"{farm}",A169),"{link}",G169))</f>
+        <f aca="false">IF(A169="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F169="ar",$B$7,$B$6)," {name}",IF(B169="",""," "&amp;B169)),"{farm}",A169),"{link}",G169))</f>
         <v/>
       </c>
       <c r="I169" s="9" t="str">
@@ -4557,7 +4940,7 @@
         <v/>
       </c>
       <c r="H170" s="9" t="str">
-        <f aca="false">IF(A170="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F170="ar",$B$7,$B$6),"{name}",IF(B170="","",B170)),"{farm}",A170),"{link}",G170))</f>
+        <f aca="false">IF(A170="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F170="ar",$B$7,$B$6)," {name}",IF(B170="",""," "&amp;B170)),"{farm}",A170),"{link}",G170))</f>
         <v/>
       </c>
       <c r="I170" s="9" t="str">
@@ -4580,7 +4963,7 @@
         <v/>
       </c>
       <c r="H171" s="9" t="str">
-        <f aca="false">IF(A171="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F171="ar",$B$7,$B$6),"{name}",IF(B171="","",B171)),"{farm}",A171),"{link}",G171))</f>
+        <f aca="false">IF(A171="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F171="ar",$B$7,$B$6)," {name}",IF(B171="",""," "&amp;B171)),"{farm}",A171),"{link}",G171))</f>
         <v/>
       </c>
       <c r="I171" s="9" t="str">
@@ -4603,7 +4986,7 @@
         <v/>
       </c>
       <c r="H172" s="9" t="str">
-        <f aca="false">IF(A172="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F172="ar",$B$7,$B$6),"{name}",IF(B172="","",B172)),"{farm}",A172),"{link}",G172))</f>
+        <f aca="false">IF(A172="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F172="ar",$B$7,$B$6)," {name}",IF(B172="",""," "&amp;B172)),"{farm}",A172),"{link}",G172))</f>
         <v/>
       </c>
       <c r="I172" s="9" t="str">
@@ -4626,7 +5009,7 @@
         <v/>
       </c>
       <c r="H173" s="9" t="str">
-        <f aca="false">IF(A173="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F173="ar",$B$7,$B$6),"{name}",IF(B173="","",B173)),"{farm}",A173),"{link}",G173))</f>
+        <f aca="false">IF(A173="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F173="ar",$B$7,$B$6)," {name}",IF(B173="",""," "&amp;B173)),"{farm}",A173),"{link}",G173))</f>
         <v/>
       </c>
       <c r="I173" s="9" t="str">
@@ -4649,7 +5032,7 @@
         <v/>
       </c>
       <c r="H174" s="9" t="str">
-        <f aca="false">IF(A174="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F174="ar",$B$7,$B$6),"{name}",IF(B174="","",B174)),"{farm}",A174),"{link}",G174))</f>
+        <f aca="false">IF(A174="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F174="ar",$B$7,$B$6)," {name}",IF(B174="",""," "&amp;B174)),"{farm}",A174),"{link}",G174))</f>
         <v/>
       </c>
       <c r="I174" s="9" t="str">
@@ -4672,7 +5055,7 @@
         <v/>
       </c>
       <c r="H175" s="9" t="str">
-        <f aca="false">IF(A175="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F175="ar",$B$7,$B$6),"{name}",IF(B175="","",B175)),"{farm}",A175),"{link}",G175))</f>
+        <f aca="false">IF(A175="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F175="ar",$B$7,$B$6)," {name}",IF(B175="",""," "&amp;B175)),"{farm}",A175),"{link}",G175))</f>
         <v/>
       </c>
       <c r="I175" s="9" t="str">
@@ -4695,7 +5078,7 @@
         <v/>
       </c>
       <c r="H176" s="9" t="str">
-        <f aca="false">IF(A176="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F176="ar",$B$7,$B$6),"{name}",IF(B176="","",B176)),"{farm}",A176),"{link}",G176))</f>
+        <f aca="false">IF(A176="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F176="ar",$B$7,$B$6)," {name}",IF(B176="",""," "&amp;B176)),"{farm}",A176),"{link}",G176))</f>
         <v/>
       </c>
       <c r="I176" s="9" t="str">
@@ -4718,7 +5101,7 @@
         <v/>
       </c>
       <c r="H177" s="9" t="str">
-        <f aca="false">IF(A177="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F177="ar",$B$7,$B$6),"{name}",IF(B177="","",B177)),"{farm}",A177),"{link}",G177))</f>
+        <f aca="false">IF(A177="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F177="ar",$B$7,$B$6)," {name}",IF(B177="",""," "&amp;B177)),"{farm}",A177),"{link}",G177))</f>
         <v/>
       </c>
       <c r="I177" s="9" t="str">
@@ -4741,7 +5124,7 @@
         <v/>
       </c>
       <c r="H178" s="9" t="str">
-        <f aca="false">IF(A178="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F178="ar",$B$7,$B$6),"{name}",IF(B178="","",B178)),"{farm}",A178),"{link}",G178))</f>
+        <f aca="false">IF(A178="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F178="ar",$B$7,$B$6)," {name}",IF(B178="",""," "&amp;B178)),"{farm}",A178),"{link}",G178))</f>
         <v/>
       </c>
       <c r="I178" s="9" t="str">
@@ -4764,7 +5147,7 @@
         <v/>
       </c>
       <c r="H179" s="9" t="str">
-        <f aca="false">IF(A179="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F179="ar",$B$7,$B$6),"{name}",IF(B179="","",B179)),"{farm}",A179),"{link}",G179))</f>
+        <f aca="false">IF(A179="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F179="ar",$B$7,$B$6)," {name}",IF(B179="",""," "&amp;B179)),"{farm}",A179),"{link}",G179))</f>
         <v/>
       </c>
       <c r="I179" s="9" t="str">
@@ -4787,7 +5170,7 @@
         <v/>
       </c>
       <c r="H180" s="9" t="str">
-        <f aca="false">IF(A180="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F180="ar",$B$7,$B$6),"{name}",IF(B180="","",B180)),"{farm}",A180),"{link}",G180))</f>
+        <f aca="false">IF(A180="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F180="ar",$B$7,$B$6)," {name}",IF(B180="",""," "&amp;B180)),"{farm}",A180),"{link}",G180))</f>
         <v/>
       </c>
       <c r="I180" s="9" t="str">
@@ -4810,7 +5193,7 @@
         <v/>
       </c>
       <c r="H181" s="9" t="str">
-        <f aca="false">IF(A181="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F181="ar",$B$7,$B$6),"{name}",IF(B181="","",B181)),"{farm}",A181),"{link}",G181))</f>
+        <f aca="false">IF(A181="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F181="ar",$B$7,$B$6)," {name}",IF(B181="",""," "&amp;B181)),"{farm}",A181),"{link}",G181))</f>
         <v/>
       </c>
       <c r="I181" s="9" t="str">
@@ -4833,7 +5216,7 @@
         <v/>
       </c>
       <c r="H182" s="9" t="str">
-        <f aca="false">IF(A182="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F182="ar",$B$7,$B$6),"{name}",IF(B182="","",B182)),"{farm}",A182),"{link}",G182))</f>
+        <f aca="false">IF(A182="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F182="ar",$B$7,$B$6)," {name}",IF(B182="",""," "&amp;B182)),"{farm}",A182),"{link}",G182))</f>
         <v/>
       </c>
       <c r="I182" s="9" t="str">
@@ -4856,7 +5239,7 @@
         <v/>
       </c>
       <c r="H183" s="9" t="str">
-        <f aca="false">IF(A183="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F183="ar",$B$7,$B$6),"{name}",IF(B183="","",B183)),"{farm}",A183),"{link}",G183))</f>
+        <f aca="false">IF(A183="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F183="ar",$B$7,$B$6)," {name}",IF(B183="",""," "&amp;B183)),"{farm}",A183),"{link}",G183))</f>
         <v/>
       </c>
       <c r="I183" s="9" t="str">
@@ -4879,7 +5262,7 @@
         <v/>
       </c>
       <c r="H184" s="9" t="str">
-        <f aca="false">IF(A184="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F184="ar",$B$7,$B$6),"{name}",IF(B184="","",B184)),"{farm}",A184),"{link}",G184))</f>
+        <f aca="false">IF(A184="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F184="ar",$B$7,$B$6)," {name}",IF(B184="",""," "&amp;B184)),"{farm}",A184),"{link}",G184))</f>
         <v/>
       </c>
       <c r="I184" s="9" t="str">
@@ -4902,7 +5285,7 @@
         <v/>
       </c>
       <c r="H185" s="9" t="str">
-        <f aca="false">IF(A185="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F185="ar",$B$7,$B$6),"{name}",IF(B185="","",B185)),"{farm}",A185),"{link}",G185))</f>
+        <f aca="false">IF(A185="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F185="ar",$B$7,$B$6)," {name}",IF(B185="",""," "&amp;B185)),"{farm}",A185),"{link}",G185))</f>
         <v/>
       </c>
       <c r="I185" s="9" t="str">
@@ -4925,7 +5308,7 @@
         <v/>
       </c>
       <c r="H186" s="9" t="str">
-        <f aca="false">IF(A186="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F186="ar",$B$7,$B$6),"{name}",IF(B186="","",B186)),"{farm}",A186),"{link}",G186))</f>
+        <f aca="false">IF(A186="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F186="ar",$B$7,$B$6)," {name}",IF(B186="",""," "&amp;B186)),"{farm}",A186),"{link}",G186))</f>
         <v/>
       </c>
       <c r="I186" s="9" t="str">
@@ -4948,7 +5331,7 @@
         <v/>
       </c>
       <c r="H187" s="9" t="str">
-        <f aca="false">IF(A187="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F187="ar",$B$7,$B$6),"{name}",IF(B187="","",B187)),"{farm}",A187),"{link}",G187))</f>
+        <f aca="false">IF(A187="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F187="ar",$B$7,$B$6)," {name}",IF(B187="",""," "&amp;B187)),"{farm}",A187),"{link}",G187))</f>
         <v/>
       </c>
       <c r="I187" s="9" t="str">
@@ -4971,7 +5354,7 @@
         <v/>
       </c>
       <c r="H188" s="9" t="str">
-        <f aca="false">IF(A188="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F188="ar",$B$7,$B$6),"{name}",IF(B188="","",B188)),"{farm}",A188),"{link}",G188))</f>
+        <f aca="false">IF(A188="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F188="ar",$B$7,$B$6)," {name}",IF(B188="",""," "&amp;B188)),"{farm}",A188),"{link}",G188))</f>
         <v/>
       </c>
       <c r="I188" s="9" t="str">
@@ -4994,7 +5377,7 @@
         <v/>
       </c>
       <c r="H189" s="9" t="str">
-        <f aca="false">IF(A189="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F189="ar",$B$7,$B$6),"{name}",IF(B189="","",B189)),"{farm}",A189),"{link}",G189))</f>
+        <f aca="false">IF(A189="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F189="ar",$B$7,$B$6)," {name}",IF(B189="",""," "&amp;B189)),"{farm}",A189),"{link}",G189))</f>
         <v/>
       </c>
       <c r="I189" s="9" t="str">
@@ -5017,7 +5400,7 @@
         <v/>
       </c>
       <c r="H190" s="9" t="str">
-        <f aca="false">IF(A190="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F190="ar",$B$7,$B$6),"{name}",IF(B190="","",B190)),"{farm}",A190),"{link}",G190))</f>
+        <f aca="false">IF(A190="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F190="ar",$B$7,$B$6)," {name}",IF(B190="",""," "&amp;B190)),"{farm}",A190),"{link}",G190))</f>
         <v/>
       </c>
       <c r="I190" s="9" t="str">
@@ -5040,7 +5423,7 @@
         <v/>
       </c>
       <c r="H191" s="9" t="str">
-        <f aca="false">IF(A191="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F191="ar",$B$7,$B$6),"{name}",IF(B191="","",B191)),"{farm}",A191),"{link}",G191))</f>
+        <f aca="false">IF(A191="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F191="ar",$B$7,$B$6)," {name}",IF(B191="",""," "&amp;B191)),"{farm}",A191),"{link}",G191))</f>
         <v/>
       </c>
       <c r="I191" s="9" t="str">
@@ -5063,7 +5446,7 @@
         <v/>
       </c>
       <c r="H192" s="9" t="str">
-        <f aca="false">IF(A192="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F192="ar",$B$7,$B$6),"{name}",IF(B192="","",B192)),"{farm}",A192),"{link}",G192))</f>
+        <f aca="false">IF(A192="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F192="ar",$B$7,$B$6)," {name}",IF(B192="",""," "&amp;B192)),"{farm}",A192),"{link}",G192))</f>
         <v/>
       </c>
       <c r="I192" s="9" t="str">
@@ -5086,7 +5469,7 @@
         <v/>
       </c>
       <c r="H193" s="9" t="str">
-        <f aca="false">IF(A193="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F193="ar",$B$7,$B$6),"{name}",IF(B193="","",B193)),"{farm}",A193),"{link}",G193))</f>
+        <f aca="false">IF(A193="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F193="ar",$B$7,$B$6)," {name}",IF(B193="",""," "&amp;B193)),"{farm}",A193),"{link}",G193))</f>
         <v/>
       </c>
       <c r="I193" s="9" t="str">
@@ -5109,7 +5492,7 @@
         <v/>
       </c>
       <c r="H194" s="9" t="str">
-        <f aca="false">IF(A194="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F194="ar",$B$7,$B$6),"{name}",IF(B194="","",B194)),"{farm}",A194),"{link}",G194))</f>
+        <f aca="false">IF(A194="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F194="ar",$B$7,$B$6)," {name}",IF(B194="",""," "&amp;B194)),"{farm}",A194),"{link}",G194))</f>
         <v/>
       </c>
       <c r="I194" s="9" t="str">
@@ -5132,7 +5515,7 @@
         <v/>
       </c>
       <c r="H195" s="9" t="str">
-        <f aca="false">IF(A195="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F195="ar",$B$7,$B$6),"{name}",IF(B195="","",B195)),"{farm}",A195),"{link}",G195))</f>
+        <f aca="false">IF(A195="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F195="ar",$B$7,$B$6)," {name}",IF(B195="",""," "&amp;B195)),"{farm}",A195),"{link}",G195))</f>
         <v/>
       </c>
       <c r="I195" s="9" t="str">
@@ -5155,7 +5538,7 @@
         <v/>
       </c>
       <c r="H196" s="9" t="str">
-        <f aca="false">IF(A196="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F196="ar",$B$7,$B$6),"{name}",IF(B196="","",B196)),"{farm}",A196),"{link}",G196))</f>
+        <f aca="false">IF(A196="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F196="ar",$B$7,$B$6)," {name}",IF(B196="",""," "&amp;B196)),"{farm}",A196),"{link}",G196))</f>
         <v/>
       </c>
       <c r="I196" s="9" t="str">
@@ -5178,7 +5561,7 @@
         <v/>
       </c>
       <c r="H197" s="9" t="str">
-        <f aca="false">IF(A197="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F197="ar",$B$7,$B$6),"{name}",IF(B197="","",B197)),"{farm}",A197),"{link}",G197))</f>
+        <f aca="false">IF(A197="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F197="ar",$B$7,$B$6)," {name}",IF(B197="",""," "&amp;B197)),"{farm}",A197),"{link}",G197))</f>
         <v/>
       </c>
       <c r="I197" s="9" t="str">
@@ -5201,7 +5584,7 @@
         <v/>
       </c>
       <c r="H198" s="9" t="str">
-        <f aca="false">IF(A198="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F198="ar",$B$7,$B$6),"{name}",IF(B198="","",B198)),"{farm}",A198),"{link}",G198))</f>
+        <f aca="false">IF(A198="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F198="ar",$B$7,$B$6)," {name}",IF(B198="",""," "&amp;B198)),"{farm}",A198),"{link}",G198))</f>
         <v/>
       </c>
       <c r="I198" s="9" t="str">
@@ -5224,7 +5607,7 @@
         <v/>
       </c>
       <c r="H199" s="9" t="str">
-        <f aca="false">IF(A199="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F199="ar",$B$7,$B$6),"{name}",IF(B199="","",B199)),"{farm}",A199),"{link}",G199))</f>
+        <f aca="false">IF(A199="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F199="ar",$B$7,$B$6)," {name}",IF(B199="",""," "&amp;B199)),"{farm}",A199),"{link}",G199))</f>
         <v/>
       </c>
       <c r="I199" s="9" t="str">
@@ -5247,7 +5630,7 @@
         <v/>
       </c>
       <c r="H200" s="9" t="str">
-        <f aca="false">IF(A200="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F200="ar",$B$7,$B$6),"{name}",IF(B200="","",B200)),"{farm}",A200),"{link}",G200))</f>
+        <f aca="false">IF(A200="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F200="ar",$B$7,$B$6)," {name}",IF(B200="",""," "&amp;B200)),"{farm}",A200),"{link}",G200))</f>
         <v/>
       </c>
       <c r="I200" s="9" t="str">
@@ -5270,7 +5653,7 @@
         <v/>
       </c>
       <c r="H201" s="9" t="str">
-        <f aca="false">IF(A201="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F201="ar",$B$7,$B$6),"{name}",IF(B201="","",B201)),"{farm}",A201),"{link}",G201))</f>
+        <f aca="false">IF(A201="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F201="ar",$B$7,$B$6)," {name}",IF(B201="",""," "&amp;B201)),"{farm}",A201),"{link}",G201))</f>
         <v/>
       </c>
       <c r="I201" s="9" t="str">
@@ -5293,7 +5676,7 @@
         <v/>
       </c>
       <c r="H202" s="9" t="str">
-        <f aca="false">IF(A202="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F202="ar",$B$7,$B$6),"{name}",IF(B202="","",B202)),"{farm}",A202),"{link}",G202))</f>
+        <f aca="false">IF(A202="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F202="ar",$B$7,$B$6)," {name}",IF(B202="",""," "&amp;B202)),"{farm}",A202),"{link}",G202))</f>
         <v/>
       </c>
       <c r="I202" s="9" t="str">
@@ -5316,7 +5699,7 @@
         <v/>
       </c>
       <c r="H203" s="9" t="str">
-        <f aca="false">IF(A203="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F203="ar",$B$7,$B$6),"{name}",IF(B203="","",B203)),"{farm}",A203),"{link}",G203))</f>
+        <f aca="false">IF(A203="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F203="ar",$B$7,$B$6)," {name}",IF(B203="",""," "&amp;B203)),"{farm}",A203),"{link}",G203))</f>
         <v/>
       </c>
       <c r="I203" s="9" t="str">
@@ -5339,7 +5722,7 @@
         <v/>
       </c>
       <c r="H204" s="9" t="str">
-        <f aca="false">IF(A204="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F204="ar",$B$7,$B$6),"{name}",IF(B204="","",B204)),"{farm}",A204),"{link}",G204))</f>
+        <f aca="false">IF(A204="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F204="ar",$B$7,$B$6)," {name}",IF(B204="",""," "&amp;B204)),"{farm}",A204),"{link}",G204))</f>
         <v/>
       </c>
       <c r="I204" s="9" t="str">
@@ -5362,7 +5745,7 @@
         <v/>
       </c>
       <c r="H205" s="9" t="str">
-        <f aca="false">IF(A205="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F205="ar",$B$7,$B$6),"{name}",IF(B205="","",B205)),"{farm}",A205),"{link}",G205))</f>
+        <f aca="false">IF(A205="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F205="ar",$B$7,$B$6)," {name}",IF(B205="",""," "&amp;B205)),"{farm}",A205),"{link}",G205))</f>
         <v/>
       </c>
       <c r="I205" s="9" t="str">
@@ -5385,7 +5768,7 @@
         <v/>
       </c>
       <c r="H206" s="9" t="str">
-        <f aca="false">IF(A206="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F206="ar",$B$7,$B$6),"{name}",IF(B206="","",B206)),"{farm}",A206),"{link}",G206))</f>
+        <f aca="false">IF(A206="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F206="ar",$B$7,$B$6)," {name}",IF(B206="",""," "&amp;B206)),"{farm}",A206),"{link}",G206))</f>
         <v/>
       </c>
       <c r="I206" s="9" t="str">
@@ -5408,7 +5791,7 @@
         <v/>
       </c>
       <c r="H207" s="9" t="str">
-        <f aca="false">IF(A207="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F207="ar",$B$7,$B$6),"{name}",IF(B207="","",B207)),"{farm}",A207),"{link}",G207))</f>
+        <f aca="false">IF(A207="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F207="ar",$B$7,$B$6)," {name}",IF(B207="",""," "&amp;B207)),"{farm}",A207),"{link}",G207))</f>
         <v/>
       </c>
       <c r="I207" s="9" t="str">
@@ -5431,7 +5814,7 @@
         <v/>
       </c>
       <c r="H208" s="9" t="str">
-        <f aca="false">IF(A208="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F208="ar",$B$7,$B$6),"{name}",IF(B208="","",B208)),"{farm}",A208),"{link}",G208))</f>
+        <f aca="false">IF(A208="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F208="ar",$B$7,$B$6)," {name}",IF(B208="",""," "&amp;B208)),"{farm}",A208),"{link}",G208))</f>
         <v/>
       </c>
       <c r="I208" s="9" t="str">
@@ -5454,7 +5837,7 @@
         <v/>
       </c>
       <c r="H209" s="9" t="str">
-        <f aca="false">IF(A209="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F209="ar",$B$7,$B$6),"{name}",IF(B209="","",B209)),"{farm}",A209),"{link}",G209))</f>
+        <f aca="false">IF(A209="","",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(F209="ar",$B$7,$B$6)," {name}",IF(B209="",""," "&amp;B209)),"{farm}",A209),"{link}",G209))</f>
         <v/>
       </c>
       <c r="I209" s="9" t="str">
@@ -5512,32 +5895,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>36</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>37</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>38</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5545,17 +5928,17 @@
     </row>
     <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5563,7 +5946,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>43</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Name decision (Thamra), farm verification, 5 new target farms
- launch-prep: A1 done (Thamra), domains to check in order, D1 done.
- target-farms: verification from search results (status, corrections,
  public decision-makers), KACST replaced by Estidamah, 5 new candidates.
- outreach sheet: corrections, Hypo-Farm as tower, 27 farms.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dm6j71QsxSkbatZyu95Fda
</commit_message>
<xml_diff>
--- a/docs/outreach-links.xlsx
+++ b/docs/outreach-links.xlsx
@@ -782,7 +782,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Hydroponic greenhouse</t>
+          <t>Vertical tower</t>
         </is>
       </c>
       <c r="H11" s="8">
@@ -805,7 +805,7 @@
       <c r="L11" s="10" t="n"/>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>A · hydroponic herb farm, Amman</t>
+          <t>A · aeroponic indoor farm, Umm Al-Amad (Amman); active</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       <c r="L12" s="10" t="n"/>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>C · IoT sensor partner, Irbid</t>
+          <t>C · IoT sensor partner, not a farm</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       <c r="L13" s="10" t="n"/>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>C · hydroponic programmes, many farms</t>
+          <t>C · partner; hydroponics programme ended 2020</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       <c r="L14" s="10" t="n"/>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>C · hydroponics programme, farm directory</t>
+          <t>C · likely inactive since 2020; use its project list as leads</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       <c r="L16" s="10" t="n"/>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>B · women-led hydroponic cooperative</t>
+          <t>B · women-led hydroponic cooperative, Dhiban (Madaba); active 2025</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       <c r="L20" s="10" t="n"/>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>B · builds/operates hydroponic farms; check Dubai vs Sharjah entity</t>
+          <t>B · Sharjah (Al Zubair), owned by SNASCO; unclear since 2023</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       <c r="L23" s="10" t="n"/>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>C · vertical farm tech supplier, partner</t>
+          <t>C · Abu Dhabi; its Growtune software overlaps with ours (competitor or integration)</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       <c r="L26" s="10" t="n"/>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>A · hydroponic greenhouses, Jeddah (Instagram)</t>
+          <t>A · greenhouses in Khulais, north of Jeddah; unclear since 2022 (Instagram)</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       <c r="L27" s="10" t="n"/>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>B · Mowreq + YesHealth JV; confirm it's open</t>
+          <t>B · Mowreq + YesHealth; opened in Riyadh, Jan 2026</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       <c r="L28" s="10" t="n"/>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>C · hot-climate greenhouse tech, partner</t>
+          <t>C · technology only since 2023 (farm sold to Pure Harvest)</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>KACST Green CEA Centre</t>
+          <t>Estidamah</t>
         </is>
       </c>
       <c r="B30" s="7" t="n"/>
@@ -1793,7 +1793,7 @@
       <c r="L30" s="10" t="n"/>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>C · national research centre</t>
+          <t>C · replaces KACST centre (not found); check before contacting</t>
         </is>
       </c>
     </row>
@@ -1850,13 +1850,33 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="n"/>
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Mama Natura Greens</t>
+        </is>
+      </c>
       <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n"/>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
       <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
-      <c r="F32" s="7" t="n"/>
-      <c r="G32" s="7" t="n"/>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Vertical tower</t>
+        </is>
+      </c>
       <c r="H32" s="8">
         <f>IF(A32="","",$B$4&amp;"/"&amp;IF(F32="","en",F32)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A32)&amp;IF(G32="Container farm","&amp;type=container",IF(G32="Hydroponic greenhouse","&amp;type=greenhouse",IF(G32="Research lab","&amp;type=lab","")))&amp;"&amp;utm_source="&amp;IF(E32="","direct",E32)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-23")</f>
         <v/>
@@ -1869,18 +1889,46 @@
         <f>IF(OR(A32="",D32=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D32,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(I32),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="K32" s="7" t="n"/>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>to contact</t>
+        </is>
+      </c>
       <c r="L32" s="10" t="n"/>
-      <c r="M32" s="7" t="n"/>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>A · 712 m² vertical farm, Dubai; opened Oct 2023</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="n"/>
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Arable</t>
+        </is>
+      </c>
       <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="n"/>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
       <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="7" t="n"/>
-      <c r="G33" s="7" t="n"/>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Hydroponic greenhouse</t>
+        </is>
+      </c>
       <c r="H33" s="8">
         <f>IF(A33="","",$B$4&amp;"/"&amp;IF(F33="","en",F33)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A33)&amp;IF(G33="Container farm","&amp;type=container",IF(G33="Hydroponic greenhouse","&amp;type=greenhouse",IF(G33="Research lab","&amp;type=lab","")))&amp;"&amp;utm_source="&amp;IF(E33="","direct",E33)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-24")</f>
         <v/>
@@ -1893,18 +1941,46 @@
         <f>IF(OR(A33="",D33=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D33,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(I33),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="K33" s="7" t="n"/>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>to contact</t>
+        </is>
+      </c>
       <c r="L33" s="10" t="n"/>
-      <c r="M33" s="7" t="n"/>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>A · hydroponic farms for Riyadh hotels; seed round Jan 2025</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="n"/>
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Janafarm (Mowreq)</t>
+        </is>
+      </c>
       <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
       <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
-      <c r="F34" s="7" t="n"/>
-      <c r="G34" s="7" t="n"/>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Vertical tower</t>
+        </is>
+      </c>
       <c r="H34" s="8">
         <f>IF(A34="","",$B$4&amp;"/"&amp;IF(F34="","en",F34)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A34)&amp;IF(G34="Container farm","&amp;type=container",IF(G34="Hydroponic greenhouse","&amp;type=greenhouse",IF(G34="Research lab","&amp;type=lab","")))&amp;"&amp;utm_source="&amp;IF(E34="","direct",E34)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-25")</f>
         <v/>
@@ -1917,18 +1993,46 @@
         <f>IF(OR(A34="",D34=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D34,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(I34),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="K34" s="7" t="n"/>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>to contact</t>
+        </is>
+      </c>
       <c r="L34" s="10" t="n"/>
-      <c r="M34" s="7" t="n"/>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t>A · vertical leafy greens, Jeddah</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n"/>
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Dava</t>
+        </is>
+      </c>
       <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n"/>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
       <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="n"/>
-      <c r="G35" s="7" t="n"/>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Hydroponic greenhouse</t>
+        </is>
+      </c>
       <c r="H35" s="8">
         <f>IF(A35="","",$B$4&amp;"/"&amp;IF(F35="","en",F35)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A35)&amp;IF(G35="Container farm","&amp;type=container",IF(G35="Hydroponic greenhouse","&amp;type=greenhouse",IF(G35="Research lab","&amp;type=lab","")))&amp;"&amp;utm_source="&amp;IF(E35="","direct",E35)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-26")</f>
         <v/>
@@ -1941,18 +2045,46 @@
         <f>IF(OR(A35="",D35=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D35,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(I35),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="K35" s="7" t="n"/>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>to contact</t>
+        </is>
+      </c>
       <c r="L35" s="10" t="n"/>
-      <c r="M35" s="7" t="n"/>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>B · hydroponic nurseries, Al Kharj</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n"/>
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Smart Acres</t>
+        </is>
+      </c>
       <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
       <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
-      <c r="F36" s="7" t="n"/>
-      <c r="G36" s="7" t="n"/>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Container farm</t>
+        </is>
+      </c>
       <c r="H36" s="8">
         <f>IF(A36="","",$B$4&amp;"/"&amp;IF(F36="","en",F36)&amp;"/demo?farm="&amp;_xlfn.ENCODEURL(A36)&amp;IF(G36="Container farm","&amp;type=container",IF(G36="Hydroponic greenhouse","&amp;type=greenhouse",IF(G36="Research lab","&amp;type=lab","")))&amp;"&amp;utm_source="&amp;IF(E36="","direct",E36)&amp;"&amp;utm_medium=outreach&amp;utm_campaign="&amp;_xlfn.ENCODEURL($B$5)&amp;"&amp;utm_content=row-27")</f>
         <v/>
@@ -1965,9 +2097,17 @@
         <f>IF(OR(A36="",D36=""),"",HYPERLINK("https://wa.me/"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(D36,"+","")," ",""),"-",""),"(","")&amp;"?text="&amp;_xlfn.ENCODEURL(I36),"Send on WhatsApp"))</f>
         <v/>
       </c>
-      <c r="K36" s="7" t="n"/>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>to contact</t>
+        </is>
+      </c>
       <c r="L36" s="10" t="n"/>
-      <c r="M36" s="7" t="n"/>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>B · container farm, Abu Dhabi; verify active first</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -6177,7 +6317,7 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>2. 22 target farms are already listed (see docs/validation/target-farms.md). Add the contact's first name and phone, or add new farms below.</t>
+          <t>2. 27 target farms are already listed (see docs/validation/target-farms.md). Add the contact's first name and phone, or add new farms below.</t>
         </is>
       </c>
     </row>

</xml_diff>